<commit_message>
Adjusting Fennel's appearing and disappearing
</commit_message>
<xml_diff>
--- a/tools/text_helper/text.xlsx
+++ b/tools/text_helper/text.xlsx
@@ -1744,157 +1744,157 @@
     <t>cart_load_error</t>
   </si>
   <si>
+    <t>largeBox</t>
+  </si>
+  <si>
+    <t>ポケモンのレポートのよみこみは{NEW}せいこうしませんでした。カートリッジを{NEW}とりはずして、もういちどさしこんで、{NEW}Aボタンをおしてください。{NEW}{NEW}あるいは、このプログラムをもうひとつの{NEW}ゲームボーイアドバンスに{NEW}てんそうするには、SELECTボタンを{NEW}おしてください。</t>
+  </si>
+  <si>
+    <t>The POKéMON save file was not loaded successfully. Please remove and reinsert the Game Pak, and then press the A button.{NEW}{NEW}Alternatively, press the SELECT button to send this program to another Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>Échec du chagement de la sauvegarde.{NEW}Retirez la cartouche puis appuyez sur A.{NEW}{NEW}Vous pouvez également appuyer sur SELECT pour envoyer ce programme à une autre Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>El archivo de guardado de POKéMON no se cargó correctamente. Por favor, retira e inserta de nuevo el cartucho y luego presiona el botón A.{NEW}{NEW}O puedes presionar el botón Select para enviar este programa a otra Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>O arquivo de salvamento de POKéMON não foi carregado corretamente. Por favor remova e reinsira o jogo, e então pressione o botão A.{NEW}Como alternativa, pressione o botão SELECT para enviar esse programa para outro Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>pulled_cart_error</t>
+  </si>
+  <si>
+    <t>ポケモンゲームは、とりはずされました。{NEW}でんげんをきって、プログラムを{NEW}さいきどうしてください。</t>
+  </si>
+  <si>
+    <t>The POKéMON game was removed. Please turn off the system and restart the program.</t>
+  </si>
+  <si>
+    <t>La cartouche a été retirée.{NEW}{NEW}Éteignez la console et redémarrez le programme.</t>
+  </si>
+  <si>
+    <t>El juego de POKéMON fue retirado. Por favor, apaga el sistema y reinicia el programa.</t>
+  </si>
+  <si>
+    <t>O jogo de POKéMON foi removido. Por favor desligue o sistema e reinicie o programa.</t>
+  </si>
+  <si>
+    <t>send_multiboot_instructions</t>
+  </si>
+  <si>
+    <t>ゲームボーイアドバンスせんよう{NEW}つうしんケーブルでこのほんたいを、{NEW}マルチブートモードにしたもうひとつの{NEW}ゲームボーイアドバンスにつなげて{NEW}ください。{NEW}{NEW}それで、もうひとつのゲームボーイ{NEW}アドバンスにポケムーバーGBのそうしんを{NEW}かいしするには、Aボタンを{NEW}おしてください。</t>
+  </si>
+  <si>
+    <t>Please connect this system to another Game Boy Advance in Multiboot mode with a Game Boy Advance Link Cable. {NEW}{NEW}Then, press the A button to begin sending Poké Transporter GB to the second Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>Connectez une autre Game Boy Advance en mode Multiboot à celle-ci avec un Câble Link pour Game Boy Advance.{NEW}{NEW}Appuyez ensuite sur A pour démarrer l’envoi de Poké Transfert GB.</t>
+  </si>
+  <si>
+    <t>Conecta este sistema a otra Game Boy Advance en modo Multiboot con un cable link de Game Boy Advance. {NEW}{NEW}Luego, presiona el botón A para comenzar a enviar Poké Transporter GB a la segunda Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>Por favor conecte esse sistema a outro Game Boy Advance no modo Multiboot através do Cabo Link de Game Boy Advance. {NEW}{NEW}Depois, pressione o botão A para começar a enviar o Poké Transporter GB para o outro Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>send_multiboot_wait</t>
+  </si>
+  <si>
+    <t>ポケムーバーGBをもうひとつの{NEW}ゲームボーイアドバンスほんたいに{NEW}そうしんちゅう。おまちください。{NEW}{NEW}Bボタンをながおしでキャンセル。</t>
+  </si>
+  <si>
+    <t>Sending Poké Transporter GB to second Game Boy Advance system. Please wait.{NEW}{NEW}Hold the B Button to cancel.</t>
+  </si>
+  <si>
+    <t>Envoi du Poké Transfert GB à l’autre Game Boy Advance.{NEW}Veuillez patienter.{NEW}{NEW}Maintenez B pour annuler.</t>
+  </si>
+  <si>
+    <t>Enviando Poké Transporter GB al segundo sistema Game Boy Advance. Por favor, espera.{NEW}{NEW}Mantén presionado el botón B para cancelar.</t>
+  </si>
+  <si>
+    <t>Enviando Poké Transporter GB para o segundo Game Boy Advance. Por favor aguarde. {NEW}{NEW}Segure o botão B para cancelar.</t>
+  </si>
+  <si>
+    <t>send_multiboot_success</t>
+  </si>
+  <si>
+    <t>{NEW}ポケムーバーGBはぶじに{NEW}そうしんされました！{NEW}このゲームボーイアドバンス{NEW}ほんたいのでんげんは{NEW}もうきってもいいです。</t>
+  </si>
+  <si>
+    <t>{NEW}Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</t>
+  </si>
+  <si>
+    <t>Poké Transfert GB envoyé avec succès!{NEW}Vous pouvez étiendre la Game Boy Advance source.</t>
+  </si>
+  <si>
+    <t>{NEW}¡Poké Transporter GB se envió con éxito! Ya puedes apagar este sistema Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>{NEW}Poké Transporter GB foi enviado com sucesso! Agora você já pode desligar esse GameBoy Advance.</t>
+  </si>
+  <si>
+    <t>send_multiboot_failure</t>
+  </si>
+  <si>
+    <t>{NEW}ポケムーバーGBそうしんちゅうに{NEW}エラーがはっせいしました。{NEW}せつめいがめんにもどってやりなおすには、{NEW}Aボタンをおしてください。</t>
+  </si>
+  <si>
+    <t>{NEW}An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</t>
+  </si>
+  <si>
+    <t>Une erreur est survenue pendant l’envoi de Poké Transfert GB.{NEW}Appuyez sur A pour revenir à l’écran d’instructions et réessayez.</t>
+  </si>
+  <si>
+    <t>{NEW}Ocurrió un error al enviar Poké Transporter GB. Presiona el botón A para volver a la pantalla de instrucciones e inténtalo de nuevo.</t>
+  </si>
+  <si>
+    <t>{NEW}Um erro ocorreu na transferência do Poké Transporter GB. Pressione o botão A para retornar para a tela de instruções e tentar novamente.</t>
+  </si>
+  <si>
+    <t>kanto_name</t>
+  </si>
+  <si>
+    <t>This is used in the Dex to show the number of Pokemon, hence the colon</t>
+  </si>
+  <si>
+    <t>カントー：</t>
+  </si>
+  <si>
+    <t>KANTO:</t>
+  </si>
+  <si>
+    <t>관동:</t>
+  </si>
+  <si>
+    <t>johto_name</t>
+  </si>
+  <si>
+    <t>Ditto ^</t>
+  </si>
+  <si>
+    <t>ジョウト：</t>
+  </si>
+  <si>
+    <t>JOHTO:</t>
+  </si>
+  <si>
+    <t>성도:</t>
+  </si>
+  <si>
+    <t>link_success</t>
+  </si>
+  <si>
     <t>mediumBox</t>
   </si>
   <si>
-    <t>ポケモンのレポートのよみこみは{NEW}せいこうしませんでした。カートリッジを{NEW}とりはずして、もういちどさしこんで、{NEW}Aボタンをおしてください。{NEW}{NEW}あるいは、このプログラムをもうひとつの{NEW}ゲームボーイアドバンスに{NEW}てんそうするには、SELECTボタンを{NEW}おしてください。</t>
-  </si>
-  <si>
-    <t>The POKéMON save file was not loaded successfully. Please remove and reinsert the Game Pak, and then press the A button.{NEW}{NEW}Alternatively, press the SELECT button to send this program to another Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>Échec du chagement de la sauvegarde.{NEW}Retirez la cartouche puis appuyez sur A.{NEW}{NEW}Vous pouvez également appuyer sur SELECT pour envoyer ce programme à une autre Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>El archivo de guardado de POKéMON no se cargó correctamente. Por favor, retira e inserta de nuevo el cartucho y luego presiona el botón A.{NEW}{NEW}O puedes presionar el botón Select para enviar este programa a otra Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>O arquivo de salvamento de POKéMON não foi carregado corretamente. Por favor remova e reinsira o jogo, e então pressione o botão A.{NEW}Como alternativa, pressione o botão SELECT para enviar esse programa para outro Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>pulled_cart_error</t>
-  </si>
-  <si>
-    <t>text_key</t>
-  </si>
-  <si>
-    <t>ポケモンゲームは、とりはずされました。{NEW}でんげんをきって、プログラムを{NEW}さいきどうしてください。</t>
-  </si>
-  <si>
-    <t>The POKéMON game was removed. Please turn off the system and restart the program.</t>
-  </si>
-  <si>
-    <t>La cartouche a été retirée.{NEW}{NEW}Éteignez la console et redémarrez le programme.</t>
-  </si>
-  <si>
-    <t>El juego de POKéMON fue retirado. Por favor, apaga el sistema y reinicia el programa.</t>
-  </si>
-  <si>
-    <t>O jogo de POKéMON foi removido. Por favor desligue o sistema e reinicie o programa.</t>
-  </si>
-  <si>
-    <t>send_multiboot_instructions</t>
-  </si>
-  <si>
-    <t>ゲームボーイアドバンスせんよう{NEW}つうしんケーブルでこのほんたいを、{NEW}マルチブートモードにしたもうひとつの{NEW}ゲームボーイアドバンスにつなげて{NEW}ください。{NEW}{NEW}それで、もうひとつのゲームボーイ{NEW}アドバンスにポケムーバーGBのそうしんを{NEW}かいしするには、Aボタンを{NEW}おしてください。</t>
-  </si>
-  <si>
-    <t>Please connect this system to another Game Boy Advance in Multiboot mode with a Game Boy Advance Link Cable. {NEW}{NEW}Then, press the A button to begin sending Poké Transporter GB to the second Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>Connectez une autre Game Boy Advance en mode Multiboot à celle-ci avec un Câble Link pour Game Boy Advance.{NEW}{NEW}Appuyez ensuite sur A pour démarrer l’envoi de Poké Transfert GB.</t>
-  </si>
-  <si>
-    <t>Conecta este sistema a otra Game Boy Advance en modo Multiboot con un cable link de Game Boy Advance. {NEW}{NEW}Luego, presiona el botón A para comenzar a enviar Poké Transporter GB a la segunda Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>Por favor conecte esse sistema a outro Game Boy Advance no modo Multiboot através do Cabo Link de Game Boy Advance. {NEW}{NEW}Depois, pressione o botão A para começar a enviar o Poké Transporter GB para o outro Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>send_multiboot_wait</t>
-  </si>
-  <si>
-    <t>ポケムーバーGBをもうひとつの{NEW}ゲームボーイアドバンスほんたいに{NEW}そうしんちゅう。おまちください。{NEW}{NEW}Bボタンをながおしでキャンセル。</t>
-  </si>
-  <si>
-    <t>Sending Poké Transporter GB to second Game Boy Advance system. Please wait.{NEW}{NEW}Hold the B Button to cancel.</t>
-  </si>
-  <si>
-    <t>Envoi du Poké Transfert GB à l’autre Game Boy Advance.{NEW}Veuillez patienter.{NEW}{NEW}Maintenez B pour annuler.</t>
-  </si>
-  <si>
-    <t>Enviando Poké Transporter GB al segundo sistema Game Boy Advance. Por favor, espera.{NEW}{NEW}Mantén presionado el botón B para cancelar.</t>
-  </si>
-  <si>
-    <t>Enviando Poké Transporter GB para o segundo Game Boy Advance. Por favor aguarde. {NEW}{NEW}Segure o botão B para cancelar.</t>
-  </si>
-  <si>
-    <t>send_multiboot_success</t>
-  </si>
-  <si>
-    <t>{NEW}ポケムーバーGBはぶじに{NEW}そうしんされました！{NEW}このゲームボーイアドバンス{NEW}ほんたいのでんげんは{NEW}もうきってもいいです。</t>
-  </si>
-  <si>
-    <t>{NEW}Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</t>
-  </si>
-  <si>
-    <t>Poké Transfert GB envoyé avec succès!{NEW}Vous pouvez étiendre la Game Boy Advance source.</t>
-  </si>
-  <si>
-    <t>{NEW}¡Poké Transporter GB se envió con éxito! Ya puedes apagar este sistema Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>{NEW}Poké Transporter GB foi enviado com sucesso! Agora você já pode desligar esse GameBoy Advance.</t>
-  </si>
-  <si>
-    <t>send_multiboot_failure</t>
-  </si>
-  <si>
-    <t>{NEW}ポケムーバーGBそうしんちゅうに{NEW}エラーがはっせいしました。{NEW}せつめいがめんにもどってやりなおすには、{NEW}Aボタンをおしてください。</t>
-  </si>
-  <si>
-    <t>{NEW}An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</t>
-  </si>
-  <si>
-    <t>Une erreur est survenue pendant l’envoi de Poké Transfert GB.{NEW}Appuyez sur A pour revenir à l’écran d’instructions et réessayez.</t>
-  </si>
-  <si>
-    <t>{NEW}Ocurrió un error al enviar Poké Transporter GB. Presiona el botón A para volver a la pantalla de instrucciones e inténtalo de nuevo.</t>
-  </si>
-  <si>
-    <t>{NEW}Um erro ocorreu na transferência do Poké Transporter GB. Pressione o botão A para retornar para a tela de instruções e tentar novamente.</t>
-  </si>
-  <si>
-    <t>kanto_name</t>
-  </si>
-  <si>
-    <t>This is used in the Dex to show the number of Pokemon, hence the colon</t>
-  </si>
-  <si>
-    <t>カントー：</t>
-  </si>
-  <si>
-    <t>KANTO:</t>
-  </si>
-  <si>
-    <t>관동:</t>
-  </si>
-  <si>
-    <t>johto_name</t>
-  </si>
-  <si>
-    <t>Ditto ^</t>
-  </si>
-  <si>
-    <t>ジョウト：</t>
-  </si>
-  <si>
-    <t>JOHTO:</t>
-  </si>
-  <si>
-    <t>성도:</t>
-  </si>
-  <si>
-    <t>link_success</t>
-  </si>
-  <si>
     <t>Extra "empty" characters (_) added to center the text</t>
   </si>
   <si>
     <t>{NEW}{CTR}せつぞくにせいこう！{nCTR}{CTR}こうかんをたいきちゅう{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Link was successful!{nCTR}{CTR}Waiting for trade{nCTR}</t>
+    <t>{NEW}{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</t>
   </si>
   <si>
     <t>{NEW}{CTR}Connexion établie!{nCTR}En attente de l’échange…</t>
@@ -1912,7 +1912,7 @@
     <t>{NEW}{CTR}せつぞくにせいこう！{nCTR}{CTR}たいせんをたいきちゅう{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Link was successful!{nCTR}{CTR}Waiting for battle{nCTR}</t>
+    <t>{NEW}{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</t>
   </si>
   <si>
     <t>{CTR}Connexion établie!{NEW}En attente du combat…{nCTR}</t>
@@ -1930,7 +1930,7 @@
     <t>{NEW}{NEW}{CTR}ゲームボーイに{nCTR}{CTR}せつぞくちゅう{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</t>
+    <t>{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</t>
   </si>
   <si>
     <t>{NEW}{CTR}Connexion à{NEW}la Game Boy…{nCTR}</t>
@@ -1948,7 +1948,7 @@
     <t>{NEW}{CTR}データをつうしんちゅう‥‥{nCTR}{CTR}おまちください！{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Transferring data...{nCTR}{CTR}please wait!{nCTR}</t>
+    <t>{NEW}{CTR}Transferring data...{NEW}please wait!{nCTR}</t>
   </si>
   <si>
     <t>{CTR}Transfert de données…{NEW}Veuillez patienter!{nCTR}</t>
@@ -7666,7 +7666,7 @@
       </c>
       <c r="E2" s="16"/>
       <c r="F2" s="16" t="str">
-        <f t="shared" ref="F2:F81" si="2">H2</f>
+        <f t="shared" ref="F2:F364" si="2">H2</f>
         <v>Hey there! I’m PROF. FENNEL. As you can see, I’m a scientist. In fact, the subject I’m researching is TRAINERS! One more line please, thanks! Now let's scroll! My dream is to collect save files of various TRAINERS, but I haven’t had any breakthroughs yet…{NEW}So in the meantime, I’ve been working on a different project with one of my old friends! In my home region, there’s a location that can make a POKéMON’s dreams into reality. This means that any other POKéMON they meet in their dreams become real! That’s fantastic, but my goal is to do the same- just with a TRAINER’s dream instead! That’s why I need your help! I want to bring as many POKéMON out of your dreams as possible! There’s just over 250 POKéMON I want to catalogue in my DREAM POKéDEX- or DREAM DEX for short. But I’ll let you keep any POKéMON- they’re from your dreams after all! One last note, save data backups are recommended- just on the off chance that something goes wrong!{NEW} I think that’s everything… whenever you’re ready to start, just let me know!</v>
       </c>
       <c r="G2" s="16" t="s">
@@ -11097,29 +11097,30 @@
         <v>557</v>
       </c>
       <c r="E82" s="23"/>
-      <c r="F82" s="23" t="s">
+      <c r="F82" s="23" t="str">
+        <f t="shared" si="2"/>
+        <v>The POKéMON game was removed. Please turn off the system and restart the program.</v>
+      </c>
+      <c r="G82" s="23" t="s">
         <v>564</v>
       </c>
-      <c r="G82" s="23" t="s">
+      <c r="H82" s="23" t="s">
         <v>565</v>
       </c>
-      <c r="H82" s="23" t="s">
+      <c r="I82" s="23" t="s">
         <v>566</v>
-      </c>
-      <c r="I82" s="23" t="s">
-        <v>567</v>
       </c>
       <c r="J82" s="23"/>
       <c r="K82" s="23"/>
       <c r="L82" s="23"/>
       <c r="M82" s="23" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="N82" s="23"/>
       <c r="O82" s="23"/>
       <c r="P82" s="23"/>
       <c r="Q82" s="23" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="83">
@@ -11131,36 +11132,36 @@
         <v>384</v>
       </c>
       <c r="C83" s="22" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D83" s="23" t="s">
         <v>557</v>
       </c>
       <c r="E83" s="23"/>
       <c r="F83" s="23" t="str">
-        <f t="shared" ref="F83:F364" si="3">H83</f>
+        <f t="shared" si="2"/>
         <v>Please connect this system to another Game Boy Advance in Multiboot mode with a Game Boy Advance Link Cable. {NEW}{NEW}Then, press the A button to begin sending Poké Transporter GB to the second Game Boy Advance.</v>
       </c>
       <c r="G83" s="23" t="s">
+        <v>570</v>
+      </c>
+      <c r="H83" s="23" t="s">
         <v>571</v>
       </c>
-      <c r="H83" s="23" t="s">
+      <c r="I83" s="23" t="s">
         <v>572</v>
-      </c>
-      <c r="I83" s="23" t="s">
-        <v>573</v>
       </c>
       <c r="J83" s="23"/>
       <c r="K83" s="23"/>
       <c r="L83" s="23"/>
       <c r="M83" s="23" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N83" s="23"/>
       <c r="O83" s="23"/>
       <c r="P83" s="23"/>
       <c r="Q83" s="23" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="84">
@@ -11172,36 +11173,36 @@
         <v>384</v>
       </c>
       <c r="C84" s="22" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D84" s="23" t="s">
         <v>557</v>
       </c>
       <c r="E84" s="23"/>
       <c r="F84" s="23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Sending Poké Transporter GB to second Game Boy Advance system. Please wait.{NEW}{NEW}Hold the B Button to cancel.</v>
       </c>
       <c r="G84" s="23" t="s">
+        <v>576</v>
+      </c>
+      <c r="H84" s="23" t="s">
         <v>577</v>
       </c>
-      <c r="H84" s="23" t="s">
+      <c r="I84" s="23" t="s">
         <v>578</v>
-      </c>
-      <c r="I84" s="23" t="s">
-        <v>579</v>
       </c>
       <c r="J84" s="23"/>
       <c r="K84" s="23"/>
       <c r="L84" s="23"/>
       <c r="M84" s="23" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="N84" s="23"/>
       <c r="O84" s="23"/>
       <c r="P84" s="23"/>
       <c r="Q84" s="23" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="85">
@@ -11213,36 +11214,36 @@
         <v>384</v>
       </c>
       <c r="C85" s="22" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D85" s="23" t="s">
         <v>557</v>
       </c>
       <c r="E85" s="23"/>
       <c r="F85" s="23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>{NEW}Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</v>
       </c>
       <c r="G85" s="23" t="s">
+        <v>582</v>
+      </c>
+      <c r="H85" s="23" t="s">
         <v>583</v>
       </c>
-      <c r="H85" s="23" t="s">
+      <c r="I85" s="23" t="s">
         <v>584</v>
-      </c>
-      <c r="I85" s="23" t="s">
-        <v>585</v>
       </c>
       <c r="J85" s="23"/>
       <c r="K85" s="23"/>
       <c r="L85" s="23"/>
       <c r="M85" s="23" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="N85" s="23"/>
       <c r="O85" s="23"/>
       <c r="P85" s="23"/>
       <c r="Q85" s="23" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="86">
@@ -11254,36 +11255,36 @@
         <v>384</v>
       </c>
       <c r="C86" s="22" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D86" s="23" t="s">
         <v>557</v>
       </c>
       <c r="E86" s="23"/>
       <c r="F86" s="23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>{NEW}An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</v>
       </c>
       <c r="G86" s="23" t="s">
+        <v>588</v>
+      </c>
+      <c r="H86" s="23" t="s">
         <v>589</v>
       </c>
-      <c r="H86" s="23" t="s">
+      <c r="I86" s="23" t="s">
         <v>590</v>
-      </c>
-      <c r="I86" s="23" t="s">
-        <v>591</v>
       </c>
       <c r="J86" s="23"/>
       <c r="K86" s="23"/>
       <c r="L86" s="23"/>
       <c r="M86" s="23" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="N86" s="23"/>
       <c r="O86" s="23"/>
       <c r="P86" s="23"/>
       <c r="Q86" s="23" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="87">
@@ -11295,46 +11296,46 @@
         <v>384</v>
       </c>
       <c r="C87" s="22" t="s">
+        <v>593</v>
+      </c>
+      <c r="D87" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="E87" s="23" t="s">
         <v>594</v>
       </c>
-      <c r="D87" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="E87" s="23" t="s">
+      <c r="F87" s="23" t="str">
+        <f t="shared" si="2"/>
+        <v>KANTO:</v>
+      </c>
+      <c r="G87" s="23" t="s">
         <v>595</v>
       </c>
-      <c r="F87" s="23" t="str">
-        <f t="shared" si="3"/>
-        <v>KANTO:</v>
-      </c>
-      <c r="G87" s="23" t="s">
+      <c r="H87" s="23" t="s">
         <v>596</v>
       </c>
-      <c r="H87" s="23" t="s">
+      <c r="I87" s="23" t="s">
+        <v>596</v>
+      </c>
+      <c r="J87" s="23" t="s">
+        <v>596</v>
+      </c>
+      <c r="K87" s="23" t="s">
+        <v>596</v>
+      </c>
+      <c r="L87" s="23" t="s">
+        <v>596</v>
+      </c>
+      <c r="M87" s="23" t="s">
+        <v>596</v>
+      </c>
+      <c r="N87" s="23" t="s">
         <v>597</v>
-      </c>
-      <c r="I87" s="23" t="s">
-        <v>597</v>
-      </c>
-      <c r="J87" s="23" t="s">
-        <v>597</v>
-      </c>
-      <c r="K87" s="23" t="s">
-        <v>597</v>
-      </c>
-      <c r="L87" s="23" t="s">
-        <v>597</v>
-      </c>
-      <c r="M87" s="23" t="s">
-        <v>597</v>
-      </c>
-      <c r="N87" s="23" t="s">
-        <v>598</v>
       </c>
       <c r="O87" s="23"/>
       <c r="P87" s="23"/>
       <c r="Q87" s="23" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="88">
@@ -11346,46 +11347,46 @@
         <v>384</v>
       </c>
       <c r="C88" s="22" t="s">
+        <v>598</v>
+      </c>
+      <c r="D88" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="E88" s="23" t="s">
         <v>599</v>
       </c>
-      <c r="D88" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="E88" s="23" t="s">
+      <c r="F88" s="23" t="str">
+        <f t="shared" si="2"/>
+        <v>JOHTO:</v>
+      </c>
+      <c r="G88" s="23" t="s">
         <v>600</v>
       </c>
-      <c r="F88" s="23" t="str">
-        <f t="shared" si="3"/>
-        <v>JOHTO:</v>
-      </c>
-      <c r="G88" s="23" t="s">
+      <c r="H88" s="23" t="s">
         <v>601</v>
       </c>
-      <c r="H88" s="23" t="s">
+      <c r="I88" s="23" t="s">
+        <v>601</v>
+      </c>
+      <c r="J88" s="23" t="s">
+        <v>601</v>
+      </c>
+      <c r="K88" s="23" t="s">
+        <v>601</v>
+      </c>
+      <c r="L88" s="23" t="s">
+        <v>601</v>
+      </c>
+      <c r="M88" s="23" t="s">
+        <v>601</v>
+      </c>
+      <c r="N88" s="23" t="s">
         <v>602</v>
-      </c>
-      <c r="I88" s="23" t="s">
-        <v>602</v>
-      </c>
-      <c r="J88" s="23" t="s">
-        <v>602</v>
-      </c>
-      <c r="K88" s="23" t="s">
-        <v>602</v>
-      </c>
-      <c r="L88" s="23" t="s">
-        <v>602</v>
-      </c>
-      <c r="M88" s="23" t="s">
-        <v>602</v>
-      </c>
-      <c r="N88" s="23" t="s">
-        <v>603</v>
       </c>
       <c r="O88" s="23"/>
       <c r="P88" s="23"/>
       <c r="Q88" s="23" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="89">
@@ -11397,17 +11398,17 @@
         <v>384</v>
       </c>
       <c r="C89" s="22" t="s">
+        <v>603</v>
+      </c>
+      <c r="D89" s="23" t="s">
         <v>604</v>
-      </c>
-      <c r="D89" s="23" t="s">
-        <v>557</v>
       </c>
       <c r="E89" s="23" t="s">
         <v>605</v>
       </c>
       <c r="F89" s="23" t="str">
-        <f t="shared" si="3"/>
-        <v>{NEW}{CTR}Link was successful!{nCTR}{CTR}Waiting for trade{nCTR}</v>
+        <f t="shared" si="2"/>
+        <v>{NEW}{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</v>
       </c>
       <c r="G89" s="23" t="s">
         <v>606</v>
@@ -11443,14 +11444,14 @@
         <v>611</v>
       </c>
       <c r="D90" s="23" t="s">
-        <v>557</v>
+        <v>604</v>
       </c>
       <c r="E90" s="23" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F90" s="23" t="str">
-        <f t="shared" si="3"/>
-        <v>{NEW}{CTR}Link was successful!{nCTR}{CTR}Waiting for battle{nCTR}</v>
+        <f t="shared" si="2"/>
+        <v>{NEW}{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</v>
       </c>
       <c r="G90" s="23" t="s">
         <v>612</v>
@@ -11486,14 +11487,14 @@
         <v>617</v>
       </c>
       <c r="D91" s="23" t="s">
-        <v>557</v>
+        <v>604</v>
       </c>
       <c r="E91" s="23" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F91" s="23" t="str">
-        <f t="shared" si="3"/>
-        <v>{NEW}{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</v>
+        <f t="shared" si="2"/>
+        <v>{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</v>
       </c>
       <c r="G91" s="23" t="s">
         <v>618</v>
@@ -11529,14 +11530,14 @@
         <v>623</v>
       </c>
       <c r="D92" s="23" t="s">
-        <v>557</v>
+        <v>604</v>
       </c>
       <c r="E92" s="23" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F92" s="23" t="str">
-        <f t="shared" si="3"/>
-        <v>{NEW}{CTR}Transferring data...{nCTR}{CTR}please wait!{nCTR}</v>
+        <f t="shared" si="2"/>
+        <v>{NEW}{CTR}Transferring data...{NEW}please wait!{nCTR}</v>
       </c>
       <c r="G92" s="23" t="s">
         <v>624</v>
@@ -11578,7 +11579,7 @@
         <v>630</v>
       </c>
       <c r="F93" s="23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>{LVL}: </v>
       </c>
       <c r="G93" s="23" t="s">
@@ -11627,7 +11628,7 @@
       </c>
       <c r="E94" s="28"/>
       <c r="F94" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Lead developer:{NEW}{NEW}The Gears of Progress</v>
       </c>
       <c r="G94" s="28" t="s">
@@ -11670,7 +11671,7 @@
       </c>
       <c r="E95" s="28"/>
       <c r="F95" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Logo and co-ideator:{NEW}-Jome{NEW}{NEW}Spritework:{NEW}-LJ Birdman</v>
       </c>
       <c r="G95" s="28" t="s">
@@ -11713,7 +11714,7 @@
       </c>
       <c r="E96" s="28"/>
       <c r="F96" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Icon Sprites: {NEW}-LuigiTKO{NEW}-GuiAbel{NEW}-SourApple{NEW}&amp; the artists from POKéMON Showdown and Crystal Clear</v>
       </c>
       <c r="G96" s="28" t="s">
@@ -11756,7 +11757,7 @@
       </c>
       <c r="E97" s="28"/>
       <c r="F97" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Remote and Arbitrary Code Execution assistance:{NEW}{NEW}-TimoVM</v>
       </c>
       <c r="G97" s="28" t="s">
@@ -11797,7 +11798,7 @@
       </c>
       <c r="E98" s="28"/>
       <c r="F98" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Development assistance:{NEW}-im a blisy{NEW}-rileyk64{NEW}-Shao</v>
       </c>
       <c r="G98" s="28" t="s">
@@ -11838,7 +11839,7 @@
       </c>
       <c r="E99" s="28"/>
       <c r="F99" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Space Optimization:{NEW}-easyaspi314{NEW}{NEW}Remote Multiboot functionality and Data Compression:{NEW}-risingPhil</v>
       </c>
       <c r="G99" s="28" t="s">
@@ -11879,7 +11880,7 @@
       </c>
       <c r="E100" s="28"/>
       <c r="F100" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Built using:{NEW}-DevkitPro{NEW}-LibTonc{NEW}-LibGBA</v>
       </c>
       <c r="G100" s="28" t="s">
@@ -11920,7 +11921,7 @@
       </c>
       <c r="E101" s="28"/>
       <c r="F101" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Inspired by the works of:{NEW}-Goppier{NEW}-Lorenzooone{NEW}-im a blisy{NEW}-RETIRE</v>
       </c>
       <c r="G101" s="28" t="s">
@@ -11961,7 +11962,7 @@
       </c>
       <c r="E102" s="28"/>
       <c r="F102" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Programs used:{NEW}-HexManiacAdvance{NEW}-PKHeX{NEW}-WC3Tool{NEW}-Usenti{NEW}-SappyMidToAGB</v>
       </c>
       <c r="G102" s="28" t="s">
@@ -12002,7 +12003,7 @@
       </c>
       <c r="E103" s="28"/>
       <c r="F103" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Open Source Code and Libraries:{NEW}-libtonc-examples{NEW}-PokemonGen3toGenX{NEW}-gba-link-connection{NEW}-awesome-gbadev{NEW}-arduino-poke-gen2</v>
       </c>
       <c r="G103" s="28" t="s">
@@ -12043,7 +12044,7 @@
       </c>
       <c r="E104" s="28"/>
       <c r="F104" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Research resources:{NEW}-arm-docs{NEW}-PokemonGen3toGenX{NEW}{NEW}Full links can be found on this program’s GitHub</v>
       </c>
       <c r="G104" s="28" t="s">
@@ -12084,7 +12085,7 @@
       </c>
       <c r="E105" s="28"/>
       <c r="F105" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ROM data obtained from decompilations created by the PRET team</v>
       </c>
       <c r="G105" s="28" t="s">
@@ -12125,7 +12126,7 @@
       </c>
       <c r="E106" s="28"/>
       <c r="F106" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>POKéMON data obtained from:{NEW}-Bulbapedia{NEW}-Serebii{NEW}-PokeAPI.com</v>
       </c>
       <c r="G106" s="28" t="s">
@@ -12166,7 +12167,7 @@
       </c>
       <c r="E107" s="28"/>
       <c r="F107" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Discord community assistance:{NEW}-Hex Maniac Advance{NEW} Development{NEW}-gbadev{NEW}-pret</v>
       </c>
       <c r="G107" s="28" t="s">
@@ -12207,7 +12208,7 @@
       </c>
       <c r="E108" s="28"/>
       <c r="F108" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Writing assistance:{NEW}-Mad</v>
       </c>
       <c r="G108" s="28" t="s">
@@ -12248,7 +12249,7 @@
       </c>
       <c r="E109" s="28"/>
       <c r="F109" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>An immense thanks to Lorenzooone for their assistance in reading &amp; writing save data. Without them, this project would not have been possible.</v>
       </c>
       <c r="G109" s="28" t="s">
@@ -12289,7 +12290,7 @@
       </c>
       <c r="E110" s="28"/>
       <c r="F110" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>Special thanks to roku, Sleepy, Eza, sarahtonin, Basabi, Mad, and everyone who has listened to me talk about this for multiple years!</v>
       </c>
       <c r="G110" s="28" t="s">
@@ -12330,7 +12331,7 @@
       </c>
       <c r="E111" s="28"/>
       <c r="F111" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>All POKéMON names, sprites, and names of related resources are copyright Nintendo, Creatures, and GAME FREAK.</v>
       </c>
       <c r="G111" s="28" t="s">
@@ -12371,7 +12372,7 @@
       </c>
       <c r="E112" s="28"/>
       <c r="F112" s="28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>This project is not endorsed or supported by GAME FREAK/Nintendo.{NEW}{NEW}Please support the original developers.</v>
       </c>
       <c r="G112" s="28" t="s">
@@ -12412,7 +12413,7 @@
       </c>
       <c r="E113" s="30"/>
       <c r="F113" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MISSINGNO.</v>
       </c>
       <c r="G113" s="30" t="s">
@@ -12459,7 +12460,7 @@
       </c>
       <c r="E114" s="30"/>
       <c r="F114" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BULBASAUR</v>
       </c>
       <c r="G114" s="30" t="s">
@@ -12508,7 +12509,7 @@
       </c>
       <c r="E115" s="30"/>
       <c r="F115" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>IVYSAUR</v>
       </c>
       <c r="G115" s="30" t="s">
@@ -12557,7 +12558,7 @@
       </c>
       <c r="E116" s="30"/>
       <c r="F116" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VENUSAUR</v>
       </c>
       <c r="G116" s="30" t="s">
@@ -12606,7 +12607,7 @@
       </c>
       <c r="E117" s="30"/>
       <c r="F117" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CHARMANDER</v>
       </c>
       <c r="G117" s="30" t="s">
@@ -12655,7 +12656,7 @@
       </c>
       <c r="E118" s="30"/>
       <c r="F118" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CHARMELEON</v>
       </c>
       <c r="G118" s="30" t="s">
@@ -12704,7 +12705,7 @@
       </c>
       <c r="E119" s="30"/>
       <c r="F119" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CHARIZARD</v>
       </c>
       <c r="G119" s="30" t="s">
@@ -12753,7 +12754,7 @@
       </c>
       <c r="E120" s="30"/>
       <c r="F120" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SQUIRTLE</v>
       </c>
       <c r="G120" s="30" t="s">
@@ -12802,7 +12803,7 @@
       </c>
       <c r="E121" s="30"/>
       <c r="F121" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WARTORTLE</v>
       </c>
       <c r="G121" s="30" t="s">
@@ -12851,7 +12852,7 @@
       </c>
       <c r="E122" s="30"/>
       <c r="F122" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BLASTOISE</v>
       </c>
       <c r="G122" s="30" t="s">
@@ -12900,7 +12901,7 @@
       </c>
       <c r="E123" s="30"/>
       <c r="F123" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CATERPIE</v>
       </c>
       <c r="G123" s="30" t="s">
@@ -12949,7 +12950,7 @@
       </c>
       <c r="E124" s="30"/>
       <c r="F124" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>METAPOD</v>
       </c>
       <c r="G124" s="30" t="s">
@@ -12998,7 +12999,7 @@
       </c>
       <c r="E125" s="30"/>
       <c r="F125" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BUTTERFREE</v>
       </c>
       <c r="G125" s="30" t="s">
@@ -13047,7 +13048,7 @@
       </c>
       <c r="E126" s="30"/>
       <c r="F126" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WEEDLE</v>
       </c>
       <c r="G126" s="30" t="s">
@@ -13096,7 +13097,7 @@
       </c>
       <c r="E127" s="30"/>
       <c r="F127" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KAKUNA</v>
       </c>
       <c r="G127" s="30" t="s">
@@ -13145,7 +13146,7 @@
       </c>
       <c r="E128" s="30"/>
       <c r="F128" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BEEDRILL</v>
       </c>
       <c r="G128" s="30" t="s">
@@ -13194,7 +13195,7 @@
       </c>
       <c r="E129" s="30"/>
       <c r="F129" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PIDGEY</v>
       </c>
       <c r="G129" s="30" t="s">
@@ -13243,7 +13244,7 @@
       </c>
       <c r="E130" s="30"/>
       <c r="F130" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PIDGEOTTO</v>
       </c>
       <c r="G130" s="30" t="s">
@@ -13292,7 +13293,7 @@
       </c>
       <c r="E131" s="30"/>
       <c r="F131" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PIDGEOT</v>
       </c>
       <c r="G131" s="30" t="s">
@@ -13341,7 +13342,7 @@
       </c>
       <c r="E132" s="30"/>
       <c r="F132" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RATTATA</v>
       </c>
       <c r="G132" s="30" t="s">
@@ -13390,7 +13391,7 @@
       </c>
       <c r="E133" s="30"/>
       <c r="F133" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RATICATE</v>
       </c>
       <c r="G133" s="30" t="s">
@@ -13439,7 +13440,7 @@
       </c>
       <c r="E134" s="30"/>
       <c r="F134" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SPEAROW</v>
       </c>
       <c r="G134" s="30" t="s">
@@ -13488,7 +13489,7 @@
       </c>
       <c r="E135" s="30"/>
       <c r="F135" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FEAROW</v>
       </c>
       <c r="G135" s="30" t="s">
@@ -13537,7 +13538,7 @@
       </c>
       <c r="E136" s="30"/>
       <c r="F136" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>EKANS</v>
       </c>
       <c r="G136" s="30" t="s">
@@ -13586,7 +13587,7 @@
       </c>
       <c r="E137" s="30"/>
       <c r="F137" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ARBOK</v>
       </c>
       <c r="G137" s="30" t="s">
@@ -13635,7 +13636,7 @@
       </c>
       <c r="E138" s="30"/>
       <c r="F138" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PIKACHU</v>
       </c>
       <c r="G138" s="30" t="s">
@@ -13684,7 +13685,7 @@
       </c>
       <c r="E139" s="30"/>
       <c r="F139" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RAICHU</v>
       </c>
       <c r="G139" s="30" t="s">
@@ -13733,7 +13734,7 @@
       </c>
       <c r="E140" s="30"/>
       <c r="F140" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SANDSHREW</v>
       </c>
       <c r="G140" s="30" t="s">
@@ -13782,7 +13783,7 @@
       </c>
       <c r="E141" s="30"/>
       <c r="F141" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SANDSLASH</v>
       </c>
       <c r="G141" s="30" t="s">
@@ -13831,7 +13832,7 @@
       </c>
       <c r="E142" s="30"/>
       <c r="F142" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NIDORAN♀</v>
       </c>
       <c r="G142" s="30" t="s">
@@ -13880,7 +13881,7 @@
       </c>
       <c r="E143" s="30"/>
       <c r="F143" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NIDORINA</v>
       </c>
       <c r="G143" s="30" t="s">
@@ -13929,7 +13930,7 @@
       </c>
       <c r="E144" s="30"/>
       <c r="F144" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NIDOQUEEN</v>
       </c>
       <c r="G144" s="30" t="s">
@@ -13978,7 +13979,7 @@
       </c>
       <c r="E145" s="30"/>
       <c r="F145" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NIDORAN♂</v>
       </c>
       <c r="G145" s="30" t="s">
@@ -14027,7 +14028,7 @@
       </c>
       <c r="E146" s="30"/>
       <c r="F146" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NIDORINO</v>
       </c>
       <c r="G146" s="30" t="s">
@@ -14076,7 +14077,7 @@
       </c>
       <c r="E147" s="30"/>
       <c r="F147" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NIDOKING</v>
       </c>
       <c r="G147" s="30" t="s">
@@ -14125,7 +14126,7 @@
       </c>
       <c r="E148" s="30"/>
       <c r="F148" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CLEFAIRY</v>
       </c>
       <c r="G148" s="30" t="s">
@@ -14174,7 +14175,7 @@
       </c>
       <c r="E149" s="30"/>
       <c r="F149" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CLEFABLE</v>
       </c>
       <c r="G149" s="30" t="s">
@@ -14223,7 +14224,7 @@
       </c>
       <c r="E150" s="30"/>
       <c r="F150" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VULPIX</v>
       </c>
       <c r="G150" s="30" t="s">
@@ -14272,7 +14273,7 @@
       </c>
       <c r="E151" s="30"/>
       <c r="F151" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NINETALES</v>
       </c>
       <c r="G151" s="30" t="s">
@@ -14321,7 +14322,7 @@
       </c>
       <c r="E152" s="30"/>
       <c r="F152" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>JIGGLYPUFF</v>
       </c>
       <c r="G152" s="30" t="s">
@@ -14370,7 +14371,7 @@
       </c>
       <c r="E153" s="30"/>
       <c r="F153" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WIGGLYTUFF</v>
       </c>
       <c r="G153" s="30" t="s">
@@ -14419,7 +14420,7 @@
       </c>
       <c r="E154" s="30"/>
       <c r="F154" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ZUBAT</v>
       </c>
       <c r="G154" s="30" t="s">
@@ -14468,7 +14469,7 @@
       </c>
       <c r="E155" s="30"/>
       <c r="F155" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GOLBAT</v>
       </c>
       <c r="G155" s="30" t="s">
@@ -14517,7 +14518,7 @@
       </c>
       <c r="E156" s="30"/>
       <c r="F156" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ODDISH</v>
       </c>
       <c r="G156" s="30" t="s">
@@ -14566,7 +14567,7 @@
       </c>
       <c r="E157" s="30"/>
       <c r="F157" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GLOOM</v>
       </c>
       <c r="G157" s="30" t="s">
@@ -14615,7 +14616,7 @@
       </c>
       <c r="E158" s="30"/>
       <c r="F158" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VILEPLUME</v>
       </c>
       <c r="G158" s="30" t="s">
@@ -14664,7 +14665,7 @@
       </c>
       <c r="E159" s="30"/>
       <c r="F159" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PARAS</v>
       </c>
       <c r="G159" s="30" t="s">
@@ -14713,7 +14714,7 @@
       </c>
       <c r="E160" s="30"/>
       <c r="F160" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PARASECT</v>
       </c>
       <c r="G160" s="30" t="s">
@@ -14762,7 +14763,7 @@
       </c>
       <c r="E161" s="30"/>
       <c r="F161" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VENONAT</v>
       </c>
       <c r="G161" s="30" t="s">
@@ -14811,7 +14812,7 @@
       </c>
       <c r="E162" s="30"/>
       <c r="F162" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VENOMOTH</v>
       </c>
       <c r="G162" s="30" t="s">
@@ -14860,7 +14861,7 @@
       </c>
       <c r="E163" s="30"/>
       <c r="F163" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DIGLETT</v>
       </c>
       <c r="G163" s="30" t="s">
@@ -14909,7 +14910,7 @@
       </c>
       <c r="E164" s="30"/>
       <c r="F164" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DUGTRIO</v>
       </c>
       <c r="G164" s="30" t="s">
@@ -14958,7 +14959,7 @@
       </c>
       <c r="E165" s="30"/>
       <c r="F165" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MEOWTH</v>
       </c>
       <c r="G165" s="30" t="s">
@@ -15007,7 +15008,7 @@
       </c>
       <c r="E166" s="30"/>
       <c r="F166" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PERSIAN</v>
       </c>
       <c r="G166" s="30" t="s">
@@ -15056,7 +15057,7 @@
       </c>
       <c r="E167" s="30"/>
       <c r="F167" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PSYDUCK</v>
       </c>
       <c r="G167" s="30" t="s">
@@ -15105,7 +15106,7 @@
       </c>
       <c r="E168" s="30"/>
       <c r="F168" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GOLDUCK</v>
       </c>
       <c r="G168" s="30" t="s">
@@ -15154,7 +15155,7 @@
       </c>
       <c r="E169" s="30"/>
       <c r="F169" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MANKEY</v>
       </c>
       <c r="G169" s="30" t="s">
@@ -15203,7 +15204,7 @@
       </c>
       <c r="E170" s="30"/>
       <c r="F170" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PRIMEAPE</v>
       </c>
       <c r="G170" s="30" t="s">
@@ -15252,7 +15253,7 @@
       </c>
       <c r="E171" s="30"/>
       <c r="F171" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GROWLITHE</v>
       </c>
       <c r="G171" s="30" t="s">
@@ -15301,7 +15302,7 @@
       </c>
       <c r="E172" s="30"/>
       <c r="F172" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ARCANINE</v>
       </c>
       <c r="G172" s="30" t="s">
@@ -15350,7 +15351,7 @@
       </c>
       <c r="E173" s="30"/>
       <c r="F173" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>POLIWAG</v>
       </c>
       <c r="G173" s="30" t="s">
@@ -15399,7 +15400,7 @@
       </c>
       <c r="E174" s="30"/>
       <c r="F174" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>POLIWHIRL</v>
       </c>
       <c r="G174" s="30" t="s">
@@ -15448,7 +15449,7 @@
       </c>
       <c r="E175" s="30"/>
       <c r="F175" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>POLIWRATH</v>
       </c>
       <c r="G175" s="30" t="s">
@@ -15497,7 +15498,7 @@
       </c>
       <c r="E176" s="30"/>
       <c r="F176" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ABRA</v>
       </c>
       <c r="G176" s="30" t="s">
@@ -15546,7 +15547,7 @@
       </c>
       <c r="E177" s="30"/>
       <c r="F177" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KADABRA</v>
       </c>
       <c r="G177" s="30" t="s">
@@ -15595,7 +15596,7 @@
       </c>
       <c r="E178" s="30"/>
       <c r="F178" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ALAKAZAM</v>
       </c>
       <c r="G178" s="30" t="s">
@@ -15644,7 +15645,7 @@
       </c>
       <c r="E179" s="30"/>
       <c r="F179" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MACHOP</v>
       </c>
       <c r="G179" s="30" t="s">
@@ -15693,7 +15694,7 @@
       </c>
       <c r="E180" s="30"/>
       <c r="F180" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MACHOKE</v>
       </c>
       <c r="G180" s="30" t="s">
@@ -15742,7 +15743,7 @@
       </c>
       <c r="E181" s="30"/>
       <c r="F181" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MACHAMP</v>
       </c>
       <c r="G181" s="30" t="s">
@@ -15791,7 +15792,7 @@
       </c>
       <c r="E182" s="30"/>
       <c r="F182" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BELLSPROUT</v>
       </c>
       <c r="G182" s="30" t="s">
@@ -15840,7 +15841,7 @@
       </c>
       <c r="E183" s="30"/>
       <c r="F183" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WEEPINBELL</v>
       </c>
       <c r="G183" s="30" t="s">
@@ -15889,7 +15890,7 @@
       </c>
       <c r="E184" s="30"/>
       <c r="F184" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VICTREEBEL</v>
       </c>
       <c r="G184" s="30" t="s">
@@ -15938,7 +15939,7 @@
       </c>
       <c r="E185" s="30"/>
       <c r="F185" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TENTACOOL</v>
       </c>
       <c r="G185" s="30" t="s">
@@ -15987,7 +15988,7 @@
       </c>
       <c r="E186" s="30"/>
       <c r="F186" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TENTACRUEL</v>
       </c>
       <c r="G186" s="30" t="s">
@@ -16036,7 +16037,7 @@
       </c>
       <c r="E187" s="30"/>
       <c r="F187" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GEODUDE</v>
       </c>
       <c r="G187" s="30" t="s">
@@ -16085,7 +16086,7 @@
       </c>
       <c r="E188" s="30"/>
       <c r="F188" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GRAVELER</v>
       </c>
       <c r="G188" s="30" t="s">
@@ -16134,7 +16135,7 @@
       </c>
       <c r="E189" s="30"/>
       <c r="F189" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GOLEM</v>
       </c>
       <c r="G189" s="30" t="s">
@@ -16183,7 +16184,7 @@
       </c>
       <c r="E190" s="30"/>
       <c r="F190" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PONYTA</v>
       </c>
       <c r="G190" s="30" t="s">
@@ -16232,7 +16233,7 @@
       </c>
       <c r="E191" s="30"/>
       <c r="F191" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RAPIDASH</v>
       </c>
       <c r="G191" s="30" t="s">
@@ -16281,7 +16282,7 @@
       </c>
       <c r="E192" s="30"/>
       <c r="F192" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SLOWPOKE</v>
       </c>
       <c r="G192" s="30" t="s">
@@ -16330,7 +16331,7 @@
       </c>
       <c r="E193" s="30"/>
       <c r="F193" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SLOWBRO</v>
       </c>
       <c r="G193" s="30" t="s">
@@ -16379,7 +16380,7 @@
       </c>
       <c r="E194" s="30"/>
       <c r="F194" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAGNEMITE</v>
       </c>
       <c r="G194" s="30" t="s">
@@ -16428,7 +16429,7 @@
       </c>
       <c r="E195" s="30"/>
       <c r="F195" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAGNETON</v>
       </c>
       <c r="G195" s="30" t="s">
@@ -16477,7 +16478,7 @@
       </c>
       <c r="E196" s="30"/>
       <c r="F196" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FARFETCH’D</v>
       </c>
       <c r="G196" s="30" t="s">
@@ -16526,7 +16527,7 @@
       </c>
       <c r="E197" s="30"/>
       <c r="F197" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DODUO</v>
       </c>
       <c r="G197" s="30" t="s">
@@ -16575,7 +16576,7 @@
       </c>
       <c r="E198" s="30"/>
       <c r="F198" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DODRIO</v>
       </c>
       <c r="G198" s="30" t="s">
@@ -16624,7 +16625,7 @@
       </c>
       <c r="E199" s="30"/>
       <c r="F199" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SEEL</v>
       </c>
       <c r="G199" s="30" t="s">
@@ -16673,7 +16674,7 @@
       </c>
       <c r="E200" s="30"/>
       <c r="F200" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DEWGONG</v>
       </c>
       <c r="G200" s="30" t="s">
@@ -16722,7 +16723,7 @@
       </c>
       <c r="E201" s="30"/>
       <c r="F201" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GRIMER</v>
       </c>
       <c r="G201" s="30" t="s">
@@ -16771,7 +16772,7 @@
       </c>
       <c r="E202" s="30"/>
       <c r="F202" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MUK</v>
       </c>
       <c r="G202" s="30" t="s">
@@ -16820,7 +16821,7 @@
       </c>
       <c r="E203" s="30"/>
       <c r="F203" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SHELLDER</v>
       </c>
       <c r="G203" s="30" t="s">
@@ -16869,7 +16870,7 @@
       </c>
       <c r="E204" s="30"/>
       <c r="F204" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CLOYSTER</v>
       </c>
       <c r="G204" s="30" t="s">
@@ -16918,7 +16919,7 @@
       </c>
       <c r="E205" s="30"/>
       <c r="F205" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GASTLY</v>
       </c>
       <c r="G205" s="30" t="s">
@@ -16967,7 +16968,7 @@
       </c>
       <c r="E206" s="30"/>
       <c r="F206" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HAUNTER</v>
       </c>
       <c r="G206" s="30" t="s">
@@ -17016,7 +17017,7 @@
       </c>
       <c r="E207" s="30"/>
       <c r="F207" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GENGAR</v>
       </c>
       <c r="G207" s="30" t="s">
@@ -17065,7 +17066,7 @@
       </c>
       <c r="E208" s="30"/>
       <c r="F208" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ONIX</v>
       </c>
       <c r="G208" s="30" t="s">
@@ -17114,7 +17115,7 @@
       </c>
       <c r="E209" s="30"/>
       <c r="F209" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DROWZEE</v>
       </c>
       <c r="G209" s="30" t="s">
@@ -17163,7 +17164,7 @@
       </c>
       <c r="E210" s="30"/>
       <c r="F210" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HYPNO</v>
       </c>
       <c r="G210" s="30" t="s">
@@ -17212,7 +17213,7 @@
       </c>
       <c r="E211" s="30"/>
       <c r="F211" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KRABBY</v>
       </c>
       <c r="G211" s="30" t="s">
@@ -17261,7 +17262,7 @@
       </c>
       <c r="E212" s="30"/>
       <c r="F212" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KINGLER</v>
       </c>
       <c r="G212" s="30" t="s">
@@ -17310,7 +17311,7 @@
       </c>
       <c r="E213" s="30"/>
       <c r="F213" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VOLTORB</v>
       </c>
       <c r="G213" s="30" t="s">
@@ -17359,7 +17360,7 @@
       </c>
       <c r="E214" s="30"/>
       <c r="F214" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ELECTRODE</v>
       </c>
       <c r="G214" s="30" t="s">
@@ -17408,7 +17409,7 @@
       </c>
       <c r="E215" s="30"/>
       <c r="F215" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>EXEGGCUTE</v>
       </c>
       <c r="G215" s="30" t="s">
@@ -17457,7 +17458,7 @@
       </c>
       <c r="E216" s="30"/>
       <c r="F216" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>EXEGGUTOR</v>
       </c>
       <c r="G216" s="30" t="s">
@@ -17506,7 +17507,7 @@
       </c>
       <c r="E217" s="30"/>
       <c r="F217" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CUBONE</v>
       </c>
       <c r="G217" s="30" t="s">
@@ -17555,7 +17556,7 @@
       </c>
       <c r="E218" s="30"/>
       <c r="F218" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAROWAK</v>
       </c>
       <c r="G218" s="30" t="s">
@@ -17604,7 +17605,7 @@
       </c>
       <c r="E219" s="30"/>
       <c r="F219" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HITMONLEE</v>
       </c>
       <c r="G219" s="30" t="s">
@@ -17653,7 +17654,7 @@
       </c>
       <c r="E220" s="30"/>
       <c r="F220" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HITMONCHAN</v>
       </c>
       <c r="G220" s="30" t="s">
@@ -17702,7 +17703,7 @@
       </c>
       <c r="E221" s="30"/>
       <c r="F221" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LICKITUNG</v>
       </c>
       <c r="G221" s="30" t="s">
@@ -17751,7 +17752,7 @@
       </c>
       <c r="E222" s="30"/>
       <c r="F222" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KOFFING</v>
       </c>
       <c r="G222" s="30" t="s">
@@ -17800,7 +17801,7 @@
       </c>
       <c r="E223" s="30"/>
       <c r="F223" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WEEZING</v>
       </c>
       <c r="G223" s="30" t="s">
@@ -17849,7 +17850,7 @@
       </c>
       <c r="E224" s="30"/>
       <c r="F224" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RHYHORN</v>
       </c>
       <c r="G224" s="30" t="s">
@@ -17898,7 +17899,7 @@
       </c>
       <c r="E225" s="30"/>
       <c r="F225" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RHYDON</v>
       </c>
       <c r="G225" s="30" t="s">
@@ -17947,7 +17948,7 @@
       </c>
       <c r="E226" s="30"/>
       <c r="F226" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CHANSEY</v>
       </c>
       <c r="G226" s="30" t="s">
@@ -17996,7 +17997,7 @@
       </c>
       <c r="E227" s="30"/>
       <c r="F227" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TANGELA</v>
       </c>
       <c r="G227" s="30" t="s">
@@ -18045,7 +18046,7 @@
       </c>
       <c r="E228" s="30"/>
       <c r="F228" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KANGASKHAN</v>
       </c>
       <c r="G228" s="30" t="s">
@@ -18094,7 +18095,7 @@
       </c>
       <c r="E229" s="30"/>
       <c r="F229" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HORSEA</v>
       </c>
       <c r="G229" s="30" t="s">
@@ -18143,7 +18144,7 @@
       </c>
       <c r="E230" s="30"/>
       <c r="F230" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SEADRA</v>
       </c>
       <c r="G230" s="30" t="s">
@@ -18192,7 +18193,7 @@
       </c>
       <c r="E231" s="30"/>
       <c r="F231" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GOLDEEN</v>
       </c>
       <c r="G231" s="30" t="s">
@@ -18241,7 +18242,7 @@
       </c>
       <c r="E232" s="30"/>
       <c r="F232" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SEAKING</v>
       </c>
       <c r="G232" s="30" t="s">
@@ -18290,7 +18291,7 @@
       </c>
       <c r="E233" s="30"/>
       <c r="F233" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>STARYU</v>
       </c>
       <c r="G233" s="30" t="s">
@@ -18339,7 +18340,7 @@
       </c>
       <c r="E234" s="30"/>
       <c r="F234" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>STARMIE</v>
       </c>
       <c r="G234" s="30" t="s">
@@ -18388,7 +18389,7 @@
       </c>
       <c r="E235" s="30"/>
       <c r="F235" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MR. MIME</v>
       </c>
       <c r="G235" s="30" t="s">
@@ -18437,7 +18438,7 @@
       </c>
       <c r="E236" s="30"/>
       <c r="F236" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SCYTHER</v>
       </c>
       <c r="G236" s="30" t="s">
@@ -18486,7 +18487,7 @@
       </c>
       <c r="E237" s="30"/>
       <c r="F237" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>JYNX</v>
       </c>
       <c r="G237" s="30" t="s">
@@ -18535,7 +18536,7 @@
       </c>
       <c r="E238" s="30"/>
       <c r="F238" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ELECTABUZZ</v>
       </c>
       <c r="G238" s="30" t="s">
@@ -18584,7 +18585,7 @@
       </c>
       <c r="E239" s="30"/>
       <c r="F239" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAGMAR</v>
       </c>
       <c r="G239" s="30" t="s">
@@ -18633,7 +18634,7 @@
       </c>
       <c r="E240" s="30"/>
       <c r="F240" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PINSIR</v>
       </c>
       <c r="G240" s="30" t="s">
@@ -18682,7 +18683,7 @@
       </c>
       <c r="E241" s="30"/>
       <c r="F241" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TAUROS</v>
       </c>
       <c r="G241" s="30" t="s">
@@ -18731,7 +18732,7 @@
       </c>
       <c r="E242" s="30"/>
       <c r="F242" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAGIKARP</v>
       </c>
       <c r="G242" s="30" t="s">
@@ -18780,7 +18781,7 @@
       </c>
       <c r="E243" s="30"/>
       <c r="F243" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GYARADOS</v>
       </c>
       <c r="G243" s="30" t="s">
@@ -18829,7 +18830,7 @@
       </c>
       <c r="E244" s="30"/>
       <c r="F244" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LAPRAS</v>
       </c>
       <c r="G244" s="30" t="s">
@@ -18878,7 +18879,7 @@
       </c>
       <c r="E245" s="30"/>
       <c r="F245" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DITTO</v>
       </c>
       <c r="G245" s="30" t="s">
@@ -18927,7 +18928,7 @@
       </c>
       <c r="E246" s="30"/>
       <c r="F246" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>EEVEE</v>
       </c>
       <c r="G246" s="30" t="s">
@@ -18976,7 +18977,7 @@
       </c>
       <c r="E247" s="30"/>
       <c r="F247" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>VAPOREON</v>
       </c>
       <c r="G247" s="30" t="s">
@@ -19025,7 +19026,7 @@
       </c>
       <c r="E248" s="30"/>
       <c r="F248" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>JOLTEON</v>
       </c>
       <c r="G248" s="30" t="s">
@@ -19074,7 +19075,7 @@
       </c>
       <c r="E249" s="30"/>
       <c r="F249" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FLAREON</v>
       </c>
       <c r="G249" s="30" t="s">
@@ -19123,7 +19124,7 @@
       </c>
       <c r="E250" s="30"/>
       <c r="F250" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PORYGON</v>
       </c>
       <c r="G250" s="30" t="s">
@@ -19172,7 +19173,7 @@
       </c>
       <c r="E251" s="30"/>
       <c r="F251" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>OMANYTE</v>
       </c>
       <c r="G251" s="30" t="s">
@@ -19221,7 +19222,7 @@
       </c>
       <c r="E252" s="30"/>
       <c r="F252" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>OMASTAR</v>
       </c>
       <c r="G252" s="30" t="s">
@@ -19270,7 +19271,7 @@
       </c>
       <c r="E253" s="30"/>
       <c r="F253" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KABUTO</v>
       </c>
       <c r="G253" s="30" t="s">
@@ -19319,7 +19320,7 @@
       </c>
       <c r="E254" s="30"/>
       <c r="F254" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KABUTOPS</v>
       </c>
       <c r="G254" s="30" t="s">
@@ -19368,7 +19369,7 @@
       </c>
       <c r="E255" s="30"/>
       <c r="F255" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>AERODACTYL</v>
       </c>
       <c r="G255" s="30" t="s">
@@ -19417,7 +19418,7 @@
       </c>
       <c r="E256" s="30"/>
       <c r="F256" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SNORLAX</v>
       </c>
       <c r="G256" s="30" t="s">
@@ -19466,7 +19467,7 @@
       </c>
       <c r="E257" s="30"/>
       <c r="F257" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ARTICUNO</v>
       </c>
       <c r="G257" s="30" t="s">
@@ -19515,7 +19516,7 @@
       </c>
       <c r="E258" s="30"/>
       <c r="F258" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ZAPDOS</v>
       </c>
       <c r="G258" s="30" t="s">
@@ -19564,7 +19565,7 @@
       </c>
       <c r="E259" s="30"/>
       <c r="F259" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MOLTRES</v>
       </c>
       <c r="G259" s="30" t="s">
@@ -19613,7 +19614,7 @@
       </c>
       <c r="E260" s="30"/>
       <c r="F260" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DRATINI</v>
       </c>
       <c r="G260" s="30" t="s">
@@ -19662,7 +19663,7 @@
       </c>
       <c r="E261" s="30"/>
       <c r="F261" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DRAGONAIR</v>
       </c>
       <c r="G261" s="30" t="s">
@@ -19711,7 +19712,7 @@
       </c>
       <c r="E262" s="30"/>
       <c r="F262" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DRAGONITE</v>
       </c>
       <c r="G262" s="30" t="s">
@@ -19760,7 +19761,7 @@
       </c>
       <c r="E263" s="30"/>
       <c r="F263" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MEWTWO</v>
       </c>
       <c r="G263" s="30" t="s">
@@ -19809,7 +19810,7 @@
       </c>
       <c r="E264" s="30"/>
       <c r="F264" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MEW</v>
       </c>
       <c r="G264" s="30" t="s">
@@ -19858,7 +19859,7 @@
       </c>
       <c r="E265" s="30"/>
       <c r="F265" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CHIKORITA</v>
       </c>
       <c r="G265" s="30" t="s">
@@ -19907,7 +19908,7 @@
       </c>
       <c r="E266" s="30"/>
       <c r="F266" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BAYLEEF</v>
       </c>
       <c r="G266" s="30" t="s">
@@ -19956,7 +19957,7 @@
       </c>
       <c r="E267" s="30"/>
       <c r="F267" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MEGANIUM</v>
       </c>
       <c r="G267" s="30" t="s">
@@ -20005,7 +20006,7 @@
       </c>
       <c r="E268" s="30"/>
       <c r="F268" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CYNDAQUIL</v>
       </c>
       <c r="G268" s="30" t="s">
@@ -20054,7 +20055,7 @@
       </c>
       <c r="E269" s="30"/>
       <c r="F269" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>QUILAVA</v>
       </c>
       <c r="G269" s="30" t="s">
@@ -20103,7 +20104,7 @@
       </c>
       <c r="E270" s="30"/>
       <c r="F270" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TYPHLOSION</v>
       </c>
       <c r="G270" s="30" t="s">
@@ -20152,7 +20153,7 @@
       </c>
       <c r="E271" s="30"/>
       <c r="F271" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TOTODILE</v>
       </c>
       <c r="G271" s="30" t="s">
@@ -20201,7 +20202,7 @@
       </c>
       <c r="E272" s="30"/>
       <c r="F272" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CROCONAW</v>
       </c>
       <c r="G272" s="30" t="s">
@@ -20250,7 +20251,7 @@
       </c>
       <c r="E273" s="30"/>
       <c r="F273" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FERALIGATR</v>
       </c>
       <c r="G273" s="30" t="s">
@@ -20299,7 +20300,7 @@
       </c>
       <c r="E274" s="30"/>
       <c r="F274" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SENTRET</v>
       </c>
       <c r="G274" s="30" t="s">
@@ -20348,7 +20349,7 @@
       </c>
       <c r="E275" s="30"/>
       <c r="F275" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FURRET</v>
       </c>
       <c r="G275" s="30" t="s">
@@ -20397,7 +20398,7 @@
       </c>
       <c r="E276" s="30"/>
       <c r="F276" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HOOTHOOT</v>
       </c>
       <c r="G276" s="30" t="s">
@@ -20446,7 +20447,7 @@
       </c>
       <c r="E277" s="30"/>
       <c r="F277" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NOCTOWL</v>
       </c>
       <c r="G277" s="30" t="s">
@@ -20495,7 +20496,7 @@
       </c>
       <c r="E278" s="30"/>
       <c r="F278" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LEDYBA</v>
       </c>
       <c r="G278" s="30" t="s">
@@ -20544,7 +20545,7 @@
       </c>
       <c r="E279" s="30"/>
       <c r="F279" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LEDIAN</v>
       </c>
       <c r="G279" s="30" t="s">
@@ -20593,7 +20594,7 @@
       </c>
       <c r="E280" s="30"/>
       <c r="F280" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SPINARAK</v>
       </c>
       <c r="G280" s="30" t="s">
@@ -20642,7 +20643,7 @@
       </c>
       <c r="E281" s="30"/>
       <c r="F281" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ARIADOS</v>
       </c>
       <c r="G281" s="30" t="s">
@@ -20691,7 +20692,7 @@
       </c>
       <c r="E282" s="30"/>
       <c r="F282" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CROBAT</v>
       </c>
       <c r="G282" s="30" t="s">
@@ -20740,7 +20741,7 @@
       </c>
       <c r="E283" s="30"/>
       <c r="F283" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CHINCHOU</v>
       </c>
       <c r="G283" s="30" t="s">
@@ -20789,7 +20790,7 @@
       </c>
       <c r="E284" s="30"/>
       <c r="F284" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LANTURN</v>
       </c>
       <c r="G284" s="30" t="s">
@@ -20838,7 +20839,7 @@
       </c>
       <c r="E285" s="30"/>
       <c r="F285" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PICHU</v>
       </c>
       <c r="G285" s="30" t="s">
@@ -20887,7 +20888,7 @@
       </c>
       <c r="E286" s="30"/>
       <c r="F286" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CLEFFA</v>
       </c>
       <c r="G286" s="30" t="s">
@@ -20936,7 +20937,7 @@
       </c>
       <c r="E287" s="30"/>
       <c r="F287" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>IGGLYBUFF</v>
       </c>
       <c r="G287" s="30" t="s">
@@ -20985,7 +20986,7 @@
       </c>
       <c r="E288" s="30"/>
       <c r="F288" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TOGEPI</v>
       </c>
       <c r="G288" s="30" t="s">
@@ -21034,7 +21035,7 @@
       </c>
       <c r="E289" s="30"/>
       <c r="F289" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TOGETIC</v>
       </c>
       <c r="G289" s="30" t="s">
@@ -21083,7 +21084,7 @@
       </c>
       <c r="E290" s="30"/>
       <c r="F290" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>NATU</v>
       </c>
       <c r="G290" s="30" t="s">
@@ -21132,7 +21133,7 @@
       </c>
       <c r="E291" s="30"/>
       <c r="F291" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>XATU</v>
       </c>
       <c r="G291" s="30" t="s">
@@ -21181,7 +21182,7 @@
       </c>
       <c r="E292" s="30"/>
       <c r="F292" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAREEP</v>
       </c>
       <c r="G292" s="30" t="s">
@@ -21230,7 +21231,7 @@
       </c>
       <c r="E293" s="30"/>
       <c r="F293" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FLAAFFY</v>
       </c>
       <c r="G293" s="30" t="s">
@@ -21279,7 +21280,7 @@
       </c>
       <c r="E294" s="30"/>
       <c r="F294" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>AMPHAROS</v>
       </c>
       <c r="G294" s="30" t="s">
@@ -21328,7 +21329,7 @@
       </c>
       <c r="E295" s="30"/>
       <c r="F295" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BELLOSSOM</v>
       </c>
       <c r="G295" s="30" t="s">
@@ -21377,7 +21378,7 @@
       </c>
       <c r="E296" s="30"/>
       <c r="F296" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MARILL</v>
       </c>
       <c r="G296" s="30" t="s">
@@ -21426,7 +21427,7 @@
       </c>
       <c r="E297" s="30"/>
       <c r="F297" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>AZUMARILL</v>
       </c>
       <c r="G297" s="30" t="s">
@@ -21475,7 +21476,7 @@
       </c>
       <c r="E298" s="30"/>
       <c r="F298" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SUDOWOODO</v>
       </c>
       <c r="G298" s="30" t="s">
@@ -21524,7 +21525,7 @@
       </c>
       <c r="E299" s="30"/>
       <c r="F299" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>POLITOED</v>
       </c>
       <c r="G299" s="30" t="s">
@@ -21573,7 +21574,7 @@
       </c>
       <c r="E300" s="30"/>
       <c r="F300" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HOPPIP</v>
       </c>
       <c r="G300" s="30" t="s">
@@ -21622,7 +21623,7 @@
       </c>
       <c r="E301" s="30"/>
       <c r="F301" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SKIPLOOM</v>
       </c>
       <c r="G301" s="30" t="s">
@@ -21671,7 +21672,7 @@
       </c>
       <c r="E302" s="30"/>
       <c r="F302" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>JUMPLUFF</v>
       </c>
       <c r="G302" s="30" t="s">
@@ -21720,7 +21721,7 @@
       </c>
       <c r="E303" s="30"/>
       <c r="F303" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>AIPOM</v>
       </c>
       <c r="G303" s="30" t="s">
@@ -21769,7 +21770,7 @@
       </c>
       <c r="E304" s="30"/>
       <c r="F304" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SUNKERN</v>
       </c>
       <c r="G304" s="30" t="s">
@@ -21818,7 +21819,7 @@
       </c>
       <c r="E305" s="30"/>
       <c r="F305" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SUNFLORA</v>
       </c>
       <c r="G305" s="30" t="s">
@@ -21867,7 +21868,7 @@
       </c>
       <c r="E306" s="30"/>
       <c r="F306" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>YANMA</v>
       </c>
       <c r="G306" s="30" t="s">
@@ -21916,7 +21917,7 @@
       </c>
       <c r="E307" s="30"/>
       <c r="F307" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WOOPER</v>
       </c>
       <c r="G307" s="30" t="s">
@@ -21965,7 +21966,7 @@
       </c>
       <c r="E308" s="30"/>
       <c r="F308" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>QUAGSIRE</v>
       </c>
       <c r="G308" s="30" t="s">
@@ -22014,7 +22015,7 @@
       </c>
       <c r="E309" s="30"/>
       <c r="F309" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ESPEON</v>
       </c>
       <c r="G309" s="30" t="s">
@@ -22063,7 +22064,7 @@
       </c>
       <c r="E310" s="30"/>
       <c r="F310" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>UMBREON</v>
       </c>
       <c r="G310" s="30" t="s">
@@ -22112,7 +22113,7 @@
       </c>
       <c r="E311" s="30"/>
       <c r="F311" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MURKROW</v>
       </c>
       <c r="G311" s="30" t="s">
@@ -22161,7 +22162,7 @@
       </c>
       <c r="E312" s="30"/>
       <c r="F312" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SLOWKING</v>
       </c>
       <c r="G312" s="30" t="s">
@@ -22210,7 +22211,7 @@
       </c>
       <c r="E313" s="30"/>
       <c r="F313" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MISDREAVUS</v>
       </c>
       <c r="G313" s="30" t="s">
@@ -22259,7 +22260,7 @@
       </c>
       <c r="E314" s="30"/>
       <c r="F314" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>UNOWN</v>
       </c>
       <c r="G314" s="30" t="s">
@@ -22308,7 +22309,7 @@
       </c>
       <c r="E315" s="30"/>
       <c r="F315" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>WOBBUFFET</v>
       </c>
       <c r="G315" s="30" t="s">
@@ -22357,7 +22358,7 @@
       </c>
       <c r="E316" s="30"/>
       <c r="F316" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GIRAFARIG</v>
       </c>
       <c r="G316" s="30" t="s">
@@ -22406,7 +22407,7 @@
       </c>
       <c r="E317" s="30"/>
       <c r="F317" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PINECO</v>
       </c>
       <c r="G317" s="30" t="s">
@@ -22455,7 +22456,7 @@
       </c>
       <c r="E318" s="30"/>
       <c r="F318" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>FORRETRESS</v>
       </c>
       <c r="G318" s="30" t="s">
@@ -22504,7 +22505,7 @@
       </c>
       <c r="E319" s="30"/>
       <c r="F319" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DUNSPARCE</v>
       </c>
       <c r="G319" s="30" t="s">
@@ -22553,7 +22554,7 @@
       </c>
       <c r="E320" s="30"/>
       <c r="F320" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GLIGAR</v>
       </c>
       <c r="G320" s="30" t="s">
@@ -22602,7 +22603,7 @@
       </c>
       <c r="E321" s="30"/>
       <c r="F321" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>STEELIX</v>
       </c>
       <c r="G321" s="30" t="s">
@@ -22651,7 +22652,7 @@
       </c>
       <c r="E322" s="30"/>
       <c r="F322" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SNUBBULL</v>
       </c>
       <c r="G322" s="30" t="s">
@@ -22700,7 +22701,7 @@
       </c>
       <c r="E323" s="30"/>
       <c r="F323" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>GRANBULL</v>
       </c>
       <c r="G323" s="30" t="s">
@@ -22749,7 +22750,7 @@
       </c>
       <c r="E324" s="30"/>
       <c r="F324" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>QWILFISH</v>
       </c>
       <c r="G324" s="30" t="s">
@@ -22798,7 +22799,7 @@
       </c>
       <c r="E325" s="30"/>
       <c r="F325" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SCIZOR</v>
       </c>
       <c r="G325" s="30" t="s">
@@ -22847,7 +22848,7 @@
       </c>
       <c r="E326" s="30"/>
       <c r="F326" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SHUCKLE</v>
       </c>
       <c r="G326" s="30" t="s">
@@ -22896,7 +22897,7 @@
       </c>
       <c r="E327" s="30"/>
       <c r="F327" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HERACROSS</v>
       </c>
       <c r="G327" s="30" t="s">
@@ -22945,7 +22946,7 @@
       </c>
       <c r="E328" s="30"/>
       <c r="F328" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SNEASEL</v>
       </c>
       <c r="G328" s="30" t="s">
@@ -22994,7 +22995,7 @@
       </c>
       <c r="E329" s="30"/>
       <c r="F329" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TEDDIURSA</v>
       </c>
       <c r="G329" s="30" t="s">
@@ -23043,7 +23044,7 @@
       </c>
       <c r="E330" s="30"/>
       <c r="F330" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>URSARING</v>
       </c>
       <c r="G330" s="30" t="s">
@@ -23092,7 +23093,7 @@
       </c>
       <c r="E331" s="30"/>
       <c r="F331" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SLUGMA</v>
       </c>
       <c r="G331" s="30" t="s">
@@ -23141,7 +23142,7 @@
       </c>
       <c r="E332" s="30"/>
       <c r="F332" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAGCARGO</v>
       </c>
       <c r="G332" s="30" t="s">
@@ -23190,7 +23191,7 @@
       </c>
       <c r="E333" s="30"/>
       <c r="F333" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SWINUB</v>
       </c>
       <c r="G333" s="30" t="s">
@@ -23239,7 +23240,7 @@
       </c>
       <c r="E334" s="30"/>
       <c r="F334" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PILOSWINE</v>
       </c>
       <c r="G334" s="30" t="s">
@@ -23288,7 +23289,7 @@
       </c>
       <c r="E335" s="30"/>
       <c r="F335" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CORSOLA</v>
       </c>
       <c r="G335" s="30" t="s">
@@ -23337,7 +23338,7 @@
       </c>
       <c r="E336" s="30"/>
       <c r="F336" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>REMORAID</v>
       </c>
       <c r="G336" s="30" t="s">
@@ -23386,7 +23387,7 @@
       </c>
       <c r="E337" s="30"/>
       <c r="F337" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>OCTILLERY</v>
       </c>
       <c r="G337" s="30" t="s">
@@ -23435,7 +23436,7 @@
       </c>
       <c r="E338" s="30"/>
       <c r="F338" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DELIBIRD</v>
       </c>
       <c r="G338" s="30" t="s">
@@ -23484,7 +23485,7 @@
       </c>
       <c r="E339" s="30"/>
       <c r="F339" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MANTINE</v>
       </c>
       <c r="G339" s="30" t="s">
@@ -23533,7 +23534,7 @@
       </c>
       <c r="E340" s="30"/>
       <c r="F340" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SKARMORY</v>
       </c>
       <c r="G340" s="30" t="s">
@@ -23582,7 +23583,7 @@
       </c>
       <c r="E341" s="30"/>
       <c r="F341" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HOUNDOUR</v>
       </c>
       <c r="G341" s="30" t="s">
@@ -23631,7 +23632,7 @@
       </c>
       <c r="E342" s="30"/>
       <c r="F342" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HOUNDOOM</v>
       </c>
       <c r="G342" s="30" t="s">
@@ -23680,7 +23681,7 @@
       </c>
       <c r="E343" s="30"/>
       <c r="F343" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>KINGDRA</v>
       </c>
       <c r="G343" s="30" t="s">
@@ -23729,7 +23730,7 @@
       </c>
       <c r="E344" s="30"/>
       <c r="F344" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PHANPY</v>
       </c>
       <c r="G344" s="30" t="s">
@@ -23778,7 +23779,7 @@
       </c>
       <c r="E345" s="30"/>
       <c r="F345" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>DONPHAN</v>
       </c>
       <c r="G345" s="30" t="s">
@@ -23827,7 +23828,7 @@
       </c>
       <c r="E346" s="30"/>
       <c r="F346" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PORYGON2</v>
       </c>
       <c r="G346" s="30" t="s">
@@ -23876,7 +23877,7 @@
       </c>
       <c r="E347" s="30"/>
       <c r="F347" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>STANTLER</v>
       </c>
       <c r="G347" s="30" t="s">
@@ -23925,7 +23926,7 @@
       </c>
       <c r="E348" s="30"/>
       <c r="F348" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SMEARGLE</v>
       </c>
       <c r="G348" s="30" t="s">
@@ -23974,7 +23975,7 @@
       </c>
       <c r="E349" s="30"/>
       <c r="F349" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TYROGUE</v>
       </c>
       <c r="G349" s="30" t="s">
@@ -24023,7 +24024,7 @@
       </c>
       <c r="E350" s="30"/>
       <c r="F350" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HITMONTOP</v>
       </c>
       <c r="G350" s="30" t="s">
@@ -24072,7 +24073,7 @@
       </c>
       <c r="E351" s="30"/>
       <c r="F351" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SMOOCHUM</v>
       </c>
       <c r="G351" s="30" t="s">
@@ -24121,7 +24122,7 @@
       </c>
       <c r="E352" s="30"/>
       <c r="F352" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ELEKID</v>
       </c>
       <c r="G352" s="30" t="s">
@@ -24170,7 +24171,7 @@
       </c>
       <c r="E353" s="30"/>
       <c r="F353" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MAGBY</v>
       </c>
       <c r="G353" s="30" t="s">
@@ -24219,7 +24220,7 @@
       </c>
       <c r="E354" s="30"/>
       <c r="F354" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>MILTANK</v>
       </c>
       <c r="G354" s="30" t="s">
@@ -24268,7 +24269,7 @@
       </c>
       <c r="E355" s="30"/>
       <c r="F355" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>BLISSEY</v>
       </c>
       <c r="G355" s="30" t="s">
@@ -24317,7 +24318,7 @@
       </c>
       <c r="E356" s="30"/>
       <c r="F356" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>RAIKOU</v>
       </c>
       <c r="G356" s="30" t="s">
@@ -24366,7 +24367,7 @@
       </c>
       <c r="E357" s="30"/>
       <c r="F357" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>ENTEI</v>
       </c>
       <c r="G357" s="30" t="s">
@@ -24415,7 +24416,7 @@
       </c>
       <c r="E358" s="30"/>
       <c r="F358" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>SUICUNE</v>
       </c>
       <c r="G358" s="30" t="s">
@@ -24464,7 +24465,7 @@
       </c>
       <c r="E359" s="30"/>
       <c r="F359" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LARVITAR</v>
       </c>
       <c r="G359" s="30" t="s">
@@ -24513,7 +24514,7 @@
       </c>
       <c r="E360" s="30"/>
       <c r="F360" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>PUPITAR</v>
       </c>
       <c r="G360" s="30" t="s">
@@ -24562,7 +24563,7 @@
       </c>
       <c r="E361" s="30"/>
       <c r="F361" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>TYRANITAR</v>
       </c>
       <c r="G361" s="30" t="s">
@@ -24611,7 +24612,7 @@
       </c>
       <c r="E362" s="30"/>
       <c r="F362" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>LUGIA</v>
       </c>
       <c r="G362" s="30" t="s">
@@ -24660,7 +24661,7 @@
       </c>
       <c r="E363" s="30"/>
       <c r="F363" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>HO-OH</v>
       </c>
       <c r="G363" s="30" t="s">
@@ -24709,7 +24710,7 @@
       </c>
       <c r="E364" s="30"/>
       <c r="F364" s="30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>CELEBI</v>
       </c>
       <c r="G364" s="30" t="s">
@@ -26618,6 +26619,35 @@
         <v>1.0</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="57" t="s">
+        <v>604</v>
+      </c>
+      <c r="B9" s="59">
+        <v>4.0</v>
+      </c>
+      <c r="C9" s="59">
+        <v>154.0</v>
+      </c>
+      <c r="D9" s="59">
+        <v>-1.0</v>
+      </c>
+      <c r="E9" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="G9" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="59">
+        <v>4.0</v>
+      </c>
+      <c r="I9" s="59">
+        <v>1.0</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixing the mulitboot load menu
</commit_message>
<xml_diff>
--- a/tools/text_helper/text.xlsx
+++ b/tools/text_helper/text.xlsx
@@ -1744,27 +1744,30 @@
     <t>cart_load_error</t>
   </si>
   <si>
+    <t>creditsBox</t>
+  </si>
+  <si>
+    <t>ポケモンのレポートのよみこみは{NEW}せいこうしませんでした。カートリッジを{NEW}とりはずして、もういちどさしこんで、{NEW}Aボタンをおしてください。{NEW}{NEW}あるいは、このプログラムをもうひとつの{NEW}ゲームボーイアドバンスに{NEW}てんそうするには、SELECTボタンを{NEW}おしてください。</t>
+  </si>
+  <si>
+    <t>The POKéMON save file was not loaded successfully. Please remove and reinsert the Game Pak, and then press the A button.{NEW}{NEW}Alternatively, press the SELECT button to send this program to another Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>Échec du chagement de la sauvegarde.{NEW}Retirez la cartouche puis appuyez sur A.{NEW}{NEW}Vous pouvez également appuyer sur SELECT pour envoyer ce programme à une autre Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>El archivo de guardado de POKéMON no se cargó correctamente. Por favor, retira e inserta de nuevo el cartucho y luego presiona el botón A.{NEW}{NEW}O puedes presionar el botón Select para enviar este programa a otra Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>O arquivo de salvamento de POKéMON não foi carregado corretamente. Por favor remova e reinsira o jogo, e então pressione o botão A.{NEW}Como alternativa, pressione o botão SELECT para enviar esse programa para outro Game Boy Advance.</t>
+  </si>
+  <si>
+    <t>pulled_cart_error</t>
+  </si>
+  <si>
     <t>largeBox</t>
   </si>
   <si>
-    <t>ポケモンのレポートのよみこみは{NEW}せいこうしませんでした。カートリッジを{NEW}とりはずして、もういちどさしこんで、{NEW}Aボタンをおしてください。{NEW}{NEW}あるいは、このプログラムをもうひとつの{NEW}ゲームボーイアドバンスに{NEW}てんそうするには、SELECTボタンを{NEW}おしてください。</t>
-  </si>
-  <si>
-    <t>The POKéMON save file was not loaded successfully. Please remove and reinsert the Game Pak, and then press the A button.{NEW}{NEW}Alternatively, press the SELECT button to send this program to another Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>Échec du chagement de la sauvegarde.{NEW}Retirez la cartouche puis appuyez sur A.{NEW}{NEW}Vous pouvez également appuyer sur SELECT pour envoyer ce programme à une autre Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>El archivo de guardado de POKéMON no se cargó correctamente. Por favor, retira e inserta de nuevo el cartucho y luego presiona el botón A.{NEW}{NEW}O puedes presionar el botón Select para enviar este programa a otra Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>O arquivo de salvamento de POKéMON não foi carregado corretamente. Por favor remova e reinsira o jogo, e então pressione o botão A.{NEW}Como alternativa, pressione o botão SELECT para enviar esse programa para outro Game Boy Advance.</t>
-  </si>
-  <si>
-    <t>pulled_cart_error</t>
-  </si>
-  <si>
     <t>ポケモンゲームは、とりはずされました。{NEW}でんげんをきって、プログラムを{NEW}さいきどうしてください。</t>
   </si>
   <si>
@@ -1979,9 +1982,6 @@
   </si>
   <si>
     <t>credits_page_1</t>
-  </si>
-  <si>
-    <t>creditsBox</t>
   </si>
   <si>
     <t>しゅにんかいはつしゃ：{NEW}{NEW}The Gears of{NEW}Progress</t>
@@ -11094,7 +11094,7 @@
         <v>563</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="E82" s="23"/>
       <c r="F82" s="23" t="str">
@@ -11102,25 +11102,25 @@
         <v>The POKéMON game was removed. Please turn off the system and restart the program.</v>
       </c>
       <c r="G82" s="23" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="H82" s="23" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="I82" s="23" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J82" s="23"/>
       <c r="K82" s="23"/>
       <c r="L82" s="23"/>
       <c r="M82" s="23" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="N82" s="23"/>
       <c r="O82" s="23"/>
       <c r="P82" s="23"/>
       <c r="Q82" s="23" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="83">
@@ -11132,7 +11132,7 @@
         <v>384</v>
       </c>
       <c r="C83" s="22" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D83" s="23" t="s">
         <v>557</v>
@@ -11143,25 +11143,25 @@
         <v>Please connect this system to another Game Boy Advance in Multiboot mode with a Game Boy Advance Link Cable. {NEW}{NEW}Then, press the A button to begin sending Poké Transporter GB to the second Game Boy Advance.</v>
       </c>
       <c r="G83" s="23" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="H83" s="23" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="I83" s="23" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J83" s="23"/>
       <c r="K83" s="23"/>
       <c r="L83" s="23"/>
       <c r="M83" s="23" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="N83" s="23"/>
       <c r="O83" s="23"/>
       <c r="P83" s="23"/>
       <c r="Q83" s="23" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
     </row>
     <row r="84">
@@ -11173,7 +11173,7 @@
         <v>384</v>
       </c>
       <c r="C84" s="22" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D84" s="23" t="s">
         <v>557</v>
@@ -11184,25 +11184,25 @@
         <v>Sending Poké Transporter GB to second Game Boy Advance system. Please wait.{NEW}{NEW}Hold the B Button to cancel.</v>
       </c>
       <c r="G84" s="23" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="H84" s="23" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="I84" s="23" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="J84" s="23"/>
       <c r="K84" s="23"/>
       <c r="L84" s="23"/>
       <c r="M84" s="23" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="N84" s="23"/>
       <c r="O84" s="23"/>
       <c r="P84" s="23"/>
       <c r="Q84" s="23" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="85">
@@ -11214,7 +11214,7 @@
         <v>384</v>
       </c>
       <c r="C85" s="22" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D85" s="23" t="s">
         <v>557</v>
@@ -11225,25 +11225,25 @@
         <v>{NEW}Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</v>
       </c>
       <c r="G85" s="23" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="H85" s="23" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="I85" s="23" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="J85" s="23"/>
       <c r="K85" s="23"/>
       <c r="L85" s="23"/>
       <c r="M85" s="23" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="N85" s="23"/>
       <c r="O85" s="23"/>
       <c r="P85" s="23"/>
       <c r="Q85" s="23" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="86">
@@ -11255,7 +11255,7 @@
         <v>384</v>
       </c>
       <c r="C86" s="22" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D86" s="23" t="s">
         <v>557</v>
@@ -11266,25 +11266,25 @@
         <v>{NEW}An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</v>
       </c>
       <c r="G86" s="23" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="H86" s="23" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="I86" s="23" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="J86" s="23"/>
       <c r="K86" s="23"/>
       <c r="L86" s="23"/>
       <c r="M86" s="23" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="N86" s="23"/>
       <c r="O86" s="23"/>
       <c r="P86" s="23"/>
       <c r="Q86" s="23" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="87">
@@ -11296,46 +11296,46 @@
         <v>384</v>
       </c>
       <c r="C87" s="22" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D87" s="23" t="s">
         <v>386</v>
       </c>
       <c r="E87" s="23" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F87" s="23" t="str">
         <f t="shared" si="2"/>
         <v>KANTO:</v>
       </c>
       <c r="G87" s="23" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="H87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="I87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="J87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="K87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="L87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="M87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="N87" s="23" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="O87" s="23"/>
       <c r="P87" s="23"/>
       <c r="Q87" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="88">
@@ -11347,46 +11347,46 @@
         <v>384</v>
       </c>
       <c r="C88" s="22" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D88" s="23" t="s">
         <v>386</v>
       </c>
       <c r="E88" s="23" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F88" s="23" t="str">
         <f t="shared" si="2"/>
         <v>JOHTO:</v>
       </c>
       <c r="G88" s="23" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="H88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="I88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="J88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="K88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="L88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="M88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="N88" s="23" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="O88" s="23"/>
       <c r="P88" s="23"/>
       <c r="Q88" s="23" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="89">
@@ -11398,38 +11398,38 @@
         <v>384</v>
       </c>
       <c r="C89" s="22" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D89" s="23" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E89" s="23" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F89" s="23" t="str">
         <f t="shared" si="2"/>
         <v>{NEW}{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</v>
       </c>
       <c r="G89" s="23" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="H89" s="23" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I89" s="23" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="J89" s="23"/>
       <c r="K89" s="23"/>
       <c r="L89" s="23"/>
       <c r="M89" s="23" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="N89" s="23"/>
       <c r="O89" s="23"/>
       <c r="P89" s="23"/>
       <c r="Q89" s="23" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="90">
@@ -11441,38 +11441,38 @@
         <v>384</v>
       </c>
       <c r="C90" s="22" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D90" s="23" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E90" s="23" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F90" s="23" t="str">
         <f t="shared" si="2"/>
         <v>{NEW}{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</v>
       </c>
       <c r="G90" s="23" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="H90" s="23" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="I90" s="23" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="J90" s="23"/>
       <c r="K90" s="23"/>
       <c r="L90" s="23"/>
       <c r="M90" s="23" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="N90" s="23"/>
       <c r="O90" s="23"/>
       <c r="P90" s="23"/>
       <c r="Q90" s="23" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
     </row>
     <row r="91">
@@ -11484,38 +11484,38 @@
         <v>384</v>
       </c>
       <c r="C91" s="22" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D91" s="23" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E91" s="23" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F91" s="23" t="str">
         <f t="shared" si="2"/>
         <v>{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</v>
       </c>
       <c r="G91" s="23" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="H91" s="23" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="I91" s="23" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="J91" s="23"/>
       <c r="K91" s="23"/>
       <c r="L91" s="23"/>
       <c r="M91" s="23" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="N91" s="23"/>
       <c r="O91" s="23"/>
       <c r="P91" s="23"/>
       <c r="Q91" s="23" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
     </row>
     <row r="92">
@@ -11527,38 +11527,38 @@
         <v>384</v>
       </c>
       <c r="C92" s="22" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D92" s="23" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E92" s="23" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="F92" s="23" t="str">
         <f t="shared" si="2"/>
         <v>{NEW}{CTR}Transferring data...{NEW}please wait!{nCTR}</v>
       </c>
       <c r="G92" s="23" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="H92" s="23" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="I92" s="23" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="J92" s="23"/>
       <c r="K92" s="23"/>
       <c r="L92" s="23"/>
       <c r="M92" s="23" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="N92" s="23"/>
       <c r="O92" s="23"/>
       <c r="P92" s="23"/>
       <c r="Q92" s="23" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
     <row r="93">
@@ -11570,46 +11570,46 @@
         <v>384</v>
       </c>
       <c r="C93" s="22" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D93" s="23" t="s">
         <v>386</v>
       </c>
       <c r="E93" s="23" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F93" s="23" t="str">
         <f t="shared" si="2"/>
         <v>{LVL}: </v>
       </c>
       <c r="G93" s="23" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="H93" s="23" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="I93" s="23" t="s">
+        <v>634</v>
+      </c>
+      <c r="J93" s="23" t="s">
         <v>633</v>
       </c>
-      <c r="J93" s="23" t="s">
-        <v>632</v>
-      </c>
       <c r="K93" s="23" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="L93" s="23" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="M93" s="23" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="N93" s="23" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="O93" s="23"/>
       <c r="P93" s="23"/>
       <c r="Q93" s="23" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="94">
@@ -11621,10 +11621,10 @@
         <v>531</v>
       </c>
       <c r="C94" s="27" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D94" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E94" s="28"/>
       <c r="F94" s="28" t="str">
@@ -11667,7 +11667,7 @@
         <v>643</v>
       </c>
       <c r="D95" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E95" s="28"/>
       <c r="F95" s="28" t="str">
@@ -11710,7 +11710,7 @@
         <v>650</v>
       </c>
       <c r="D96" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E96" s="28"/>
       <c r="F96" s="28" t="str">
@@ -11753,7 +11753,7 @@
         <v>657</v>
       </c>
       <c r="D97" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E97" s="28"/>
       <c r="F97" s="28" t="str">
@@ -11794,7 +11794,7 @@
         <v>663</v>
       </c>
       <c r="D98" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E98" s="28"/>
       <c r="F98" s="28" t="str">
@@ -11835,7 +11835,7 @@
         <v>669</v>
       </c>
       <c r="D99" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E99" s="28"/>
       <c r="F99" s="28" t="str">
@@ -11876,7 +11876,7 @@
         <v>675</v>
       </c>
       <c r="D100" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E100" s="28"/>
       <c r="F100" s="28" t="str">
@@ -11917,7 +11917,7 @@
         <v>681</v>
       </c>
       <c r="D101" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E101" s="28"/>
       <c r="F101" s="28" t="str">
@@ -11958,7 +11958,7 @@
         <v>687</v>
       </c>
       <c r="D102" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E102" s="28"/>
       <c r="F102" s="28" t="str">
@@ -11999,7 +11999,7 @@
         <v>693</v>
       </c>
       <c r="D103" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E103" s="28"/>
       <c r="F103" s="28" t="str">
@@ -12040,7 +12040,7 @@
         <v>699</v>
       </c>
       <c r="D104" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E104" s="28"/>
       <c r="F104" s="28" t="str">
@@ -12081,7 +12081,7 @@
         <v>704</v>
       </c>
       <c r="D105" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E105" s="28"/>
       <c r="F105" s="28" t="str">
@@ -12122,7 +12122,7 @@
         <v>710</v>
       </c>
       <c r="D106" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E106" s="28"/>
       <c r="F106" s="28" t="str">
@@ -12163,7 +12163,7 @@
         <v>716</v>
       </c>
       <c r="D107" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E107" s="28"/>
       <c r="F107" s="28" t="str">
@@ -12204,7 +12204,7 @@
         <v>722</v>
       </c>
       <c r="D108" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E108" s="28"/>
       <c r="F108" s="28" t="str">
@@ -12245,7 +12245,7 @@
         <v>728</v>
       </c>
       <c r="D109" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E109" s="28"/>
       <c r="F109" s="28" t="str">
@@ -12286,7 +12286,7 @@
         <v>734</v>
       </c>
       <c r="D110" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E110" s="28"/>
       <c r="F110" s="28" t="str">
@@ -12327,7 +12327,7 @@
         <v>740</v>
       </c>
       <c r="D111" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E111" s="28"/>
       <c r="F111" s="28" t="str">
@@ -12368,7 +12368,7 @@
         <v>746</v>
       </c>
       <c r="D112" s="28" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="E112" s="28"/>
       <c r="F112" s="28" t="str">
@@ -26221,7 +26221,7 @@
         <v>1965</v>
       </c>
       <c r="D28" s="51" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G28" s="53" t="s">
         <v>2222</v>
@@ -26563,7 +26563,7 @@
     </row>
     <row r="7">
       <c r="A7" s="57" t="s">
-        <v>636</v>
+        <v>557</v>
       </c>
       <c r="B7" s="59">
         <v>8.0</v>
@@ -26592,7 +26592,7 @@
     </row>
     <row r="8">
       <c r="A8" s="57" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="B8" s="59">
         <v>6.0</v>
@@ -26621,7 +26621,7 @@
     </row>
     <row r="9">
       <c r="A9" s="57" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B9" s="59">
         <v>4.0</v>

</xml_diff>

<commit_message>
Fixing some text engine bugs
</commit_message>
<xml_diff>
--- a/tools/text_helper/text.xlsx
+++ b/tools/text_helper/text.xlsx
@@ -155,7 +155,7 @@
     <t>ヤッホー！　アタシはマコモ。ごらんのとおりの{NEW}けんきゅうかよ。{NEW}ちなみに、けんきゅうしているのはトレーナーについてなの！{CLR}アタシのゆめは、いろんなトレーナーのレポートを{NEW}あつめることだけどね、おおきなしんぽはまだないの‥‥{CLR}だからね、それまでは、アタシはむかしのともだちとほかの{NEW}プロジェクトにとりくんでいる！{CLR}アタシのじもとのちほうには、ポケモンのゆめをげんじつの{NEW}かたちにできるばしょがあるの。{CLR}ということは、ゆめのなかでほかにであうポケモンは{NEW}げんじつになるのよ！{CLR}すごいことなの。でもね、アタシのもくひょうはおなじことを{NEW}することなの、ただトレーナーのゆめをかわりにね！{NEW}だからアナタのてだすけがひつようなの！{CLR}アナタのゆめからポケモンをできるだけおおく{NEW}ひきだしたいのよ！{CLR}アタシのゆめのポケモンずかん、りゃくして、ゆめずかんに{NEW}とうろくしたいポケモンは、250ひきあまりいるの。{CLR}でも、でるポケモンはなんでもアナタにもたせてあげるね。{NEW}だって、けっきょくアナタのゆめからくるのね！{CLR}さいごにひとつなんだけどね、レポートのバックアップを{NEW}オススメするわよ。まんがいちにそなえて、なにかもんだいが{NEW}あったらね！{CLR}これですべてかなーとおもう‥‥　はじめるじゅんびが{NEW}できたら、いつでもアタシにしらせてね！</t>
   </si>
   <si>
-    <t>Hey there! I’m PROF. FENNEL. As you can see, I’m a scientist. In fact, the subject I’m researching is TRAINERS! One more line please, thanks! Now let's scroll! My dream is to collect save files of various TRAINERS, but I haven’t had any breakthroughs yet…{NEW}So in the meantime, I’ve been working on a different project with one of my old friends! In my home region, there’s a location that can make a POKéMON’s dreams into reality. This means that any other POKéMON they meet in their dreams become real! That’s fantastic, but my goal is to do the same- just with a TRAINER’s dream instead! That’s why I need your help! I want to bring as many POKéMON out of your dreams as possible! There’s just over 250 POKéMON I want to catalogue in my DREAM POKéDEX- or DREAM DEX for short. But I’ll let you keep any POKéMON- they’re from your dreams after all! One last note, save data backups are recommended- just on the off chance that something goes wrong!{NEW} I think that’s everything… whenever you’re ready to start, just let me know!</t>
+    <t>Hey there! I’m PROF. FENNEL. As you can see, I’m a scientist. In fact, the subject I’m researching is TRAINERS! My dream is to collect save files of various TRAINERS, but I haven’t had any breakthroughs yet…{NEW}So in the meantime, I’ve been working on a different project with one of my old friends! In my home region, there’s a location that can make a POKéMON’s dreams into reality. This means that any other POKéMON they meet in their dreams become real! That’s fantastic, but my goal is to do the same- just with a TRAINER’s dream instead! That’s why I need your help! I want to bring as many POKéMON out of your dreams as possible! There’s just over 250 POKéMON I want to catalogue in my DREAM POKéDEX- or DREAM DEX for short. But I’ll let you keep any POKéMON- they’re from your dreams after all! One last note, save data backups are recommended- just on the off chance that something goes wrong!{NEW} I think that’s everything… whenever you’re ready to start, just let me know!</t>
   </si>
   <si>
     <t>Saluuut! Je me présente: ORYSE!{NEW}Une scientifique, comme tu peux le voir.{NEW}Et ma spécialité, c’est les DRESSEURS!{NEW}Mon rêve est de réunir les sauvegardes de DRESSEURS, mais je n’ai toujours fais aucune découverte…{NEW}Du coup en attendant, j’ai travaillé sur un autre projet avec une vieille connaissance!Là d’où je viens, il y a un lieu qui matérialise les rêves des POKéMON. Faisant que chaque POKéMON qu’ils y rencontraient devenait réel! C’est méga cool, mais aujourd’hui mon but est de parvenir à la même chose avec ceux des DRESSEURS. Et c’est là que t’interviens!{NEW}Je voudais extraitre des rêves autant de POKéMON que possible! Il y a à peu près 250 POKéMON que je voudrais répertorier dans mon POKéDEX onirique, ou ONIRIDEX pour faire court. Bien entendu tu pourras garder tous les POKéMON que t’y rencontreras, ce sont les tiens après tout! Oh, une dernière chose, les backups de sauvegardes sont recommandées, juste au cas où quelque chose tourne mal! Bon, je pense que tout est prêt… Dis-moi quand tu l’es aussi!</t>
@@ -285,7 +285,7 @@
     <t>もうひとつのゲームボーイシリーズのほんたいでは、{NEW}てんそうもとのゲームボーイのポケモンゲームを{NEW}きどうしてください。{CLR}ゲームボーイのポケモンゲームでは、いまのボックスを{NEW}てんそうもとのボックスにしてね。{CLR}つぎに、もうひとつのゲームボーイシリーズのほんたいに{NEW}このゲームボーイアドバンスをゲームボーイカラーせんよう{NEW}つうしんケーブルでつなげてね。{CLR}じゅんびができたら、このデバイスでAボタンをおして、{NEW}つうしんケーブルクラブのうけつけスタッフとはなして、{NEW}それで、つうしんをかいししてね。</t>
   </si>
   <si>
-    <t>On a second Game Boy family system, please load the Game Boy POKéMON game you wish to transfer from. In your Game Boy POKéMON game, make your current box the one you want to transfer from. Then connect this Game Boy Advance to the other Game Boy family system using a Game Boy Color Link Cable. Once you’re ready, press A on this device, talk to the Cable Club attendant, and then initiate the connection.</t>
+    <t>On a second Game Boy family system, please load the Game Boy POKéMON game you wish to transfer from. In your Game Boy POKéMON game, make your current box the one you want to transfer from. Then connect this Game Boy Advance to the other Game Boy family system using a Game Boy Color Link Cable. Once you’re ready, talk to the Cable Club attendant and initiate the connection.</t>
   </si>
   <si>
     <t>Sur une autre Game Boy, peu importe le modèle, allume la version source que tu m’as indiquée précédemment.{NEW}Dans cette même version, veille aussi à ce que la BOITE active du PC soit bien celle que tu désires transférer. Ensuite, connecte les deux consoles avec un Câble Link de Game Boy Color. Enfin, dès que tout est prêt, va parler à l’hôtesse du Club Link et lance la connexion.</t>
@@ -663,7 +663,7 @@
     <t>‥‥アナタのポケモンのなかのいっひきが、てんそうきかいに{NEW}じゃましているようなの‥‥{CLR}でもね、ただのグラフィックスのもんだいにみえるから、{NEW}さきにすすめるのよ！</t>
   </si>
   <si>
-    <t>…It seems like one of your POKéMON is messing with the machine… It looks to only be graphical though, so we can continue!</t>
+    <t>…It seems like one of your POKéMON is messing with the machine! It looks to only be graphical though, so we can continue!</t>
   </si>
   <si>
     <t>… Un de tes POKéMON met le souk dans la machine… Mais le souci n’a l’air que graphique, alors continuons!</t>
@@ -7667,7 +7667,7 @@
       <c r="E2" s="16"/>
       <c r="F2" s="16" t="str">
         <f t="shared" ref="F2:F364" si="2">H2</f>
-        <v>Hey there! I’m PROF. FENNEL. As you can see, I’m a scientist. In fact, the subject I’m researching is TRAINERS! One more line please, thanks! Now let's scroll! My dream is to collect save files of various TRAINERS, but I haven’t had any breakthroughs yet…{NEW}So in the meantime, I’ve been working on a different project with one of my old friends! In my home region, there’s a location that can make a POKéMON’s dreams into reality. This means that any other POKéMON they meet in their dreams become real! That’s fantastic, but my goal is to do the same- just with a TRAINER’s dream instead! That’s why I need your help! I want to bring as many POKéMON out of your dreams as possible! There’s just over 250 POKéMON I want to catalogue in my DREAM POKéDEX- or DREAM DEX for short. But I’ll let you keep any POKéMON- they’re from your dreams after all! One last note, save data backups are recommended- just on the off chance that something goes wrong!{NEW} I think that’s everything… whenever you’re ready to start, just let me know!</v>
+        <v>Hey there! I’m PROF. FENNEL. As you can see, I’m a scientist. In fact, the subject I’m researching is TRAINERS! My dream is to collect save files of various TRAINERS, but I haven’t had any breakthroughs yet…{NEW}So in the meantime, I’ve been working on a different project with one of my old friends! In my home region, there’s a location that can make a POKéMON’s dreams into reality. This means that any other POKéMON they meet in their dreams become real! That’s fantastic, but my goal is to do the same- just with a TRAINER’s dream instead! That’s why I need your help! I want to bring as many POKéMON out of your dreams as possible! There’s just over 250 POKéMON I want to catalogue in my DREAM POKéDEX- or DREAM DEX for short. But I’ll let you keep any POKéMON- they’re from your dreams after all! One last note, save data backups are recommended- just on the off chance that something goes wrong!{NEW} I think that’s everything… whenever you’re ready to start, just let me know!</v>
       </c>
       <c r="G2" s="16" t="s">
         <v>36</v>
@@ -7880,7 +7880,7 @@
       <c r="E7" s="16"/>
       <c r="F7" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>On a second Game Boy family system, please load the Game Boy POKéMON game you wish to transfer from. In your Game Boy POKéMON game, make your current box the one you want to transfer from. Then connect this Game Boy Advance to the other Game Boy family system using a Game Boy Color Link Cable. Once you’re ready, press A on this device, talk to the Cable Club attendant, and then initiate the connection.</v>
+        <v>On a second Game Boy family system, please load the Game Boy POKéMON game you wish to transfer from. In your Game Boy POKéMON game, make your current box the one you want to transfer from. Then connect this Game Boy Advance to the other Game Boy family system using a Game Boy Color Link Cable. Once you’re ready, talk to the Cable Club attendant and initiate the connection.</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>70</v>
@@ -8741,7 +8741,7 @@
       <c r="E28" s="16"/>
       <c r="F28" s="16" t="str">
         <f t="shared" si="2"/>
-        <v>…It seems like one of your POKéMON is messing with the machine… It looks to only be graphical though, so we can continue!</v>
+        <v>…It seems like one of your POKéMON is messing with the machine! It looks to only be graphical though, so we can continue!</v>
       </c>
       <c r="G28" s="16" t="s">
         <v>196</v>

</xml_diff>

<commit_message>
Some final text modifications
</commit_message>
<xml_diff>
--- a/tools/text_helper/text.xlsx
+++ b/tools/text_helper/text.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4263" uniqueCount="2243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4264" uniqueCount="2244">
   <si>
     <r>
       <rPr>
@@ -1825,7 +1825,7 @@
     <t>{NEW}ポケムーバーGBはぶじに{NEW}そうしんされました！{NEW}このゲームボーイアドバンス{NEW}ほんたいのでんげんは{NEW}もうきってもいいです。</t>
   </si>
   <si>
-    <t>{NEW}Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</t>
+    <t>Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</t>
   </si>
   <si>
     <t>Poké Transfert GB envoyé avec succès!{NEW}Vous pouvez étiendre la Game Boy Advance source.</t>
@@ -1843,7 +1843,7 @@
     <t>{NEW}ポケムーバーGBそうしんちゅうに{NEW}エラーがはっせいしました。{NEW}せつめいがめんにもどってやりなおすには、{NEW}Aボタンをおしてください。</t>
   </si>
   <si>
-    <t>{NEW}An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</t>
+    <t>An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</t>
   </si>
   <si>
     <t>Une erreur est survenue pendant l’envoi de Poké Transfert GB.{NEW}Appuyez sur A pour revenir à l’écran d’instructions et réessayez.</t>
@@ -1897,7 +1897,7 @@
     <t>{NEW}{CTR}せつぞくにせいこう！{nCTR}{CTR}こうかんをたいきちゅう{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</t>
+    <t>{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</t>
   </si>
   <si>
     <t>{NEW}{CTR}Connexion établie!{nCTR}En attente de l’échange…</t>
@@ -1915,7 +1915,7 @@
     <t>{NEW}{CTR}せつぞくにせいこう！{nCTR}{CTR}たいせんをたいきちゅう{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</t>
+    <t>{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</t>
   </si>
   <si>
     <t>{CTR}Connexion établie!{NEW}En attente du combat…{nCTR}</t>
@@ -1933,7 +1933,7 @@
     <t>{NEW}{NEW}{CTR}ゲームボーイに{nCTR}{CTR}せつぞくちゅう{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</t>
+    <t>{CTR}Connecting to{NEW}Game Boy{nCTR}</t>
   </si>
   <si>
     <t>{NEW}{CTR}Connexion à{NEW}la Game Boy…{nCTR}</t>
@@ -1951,7 +1951,7 @@
     <t>{NEW}{CTR}データをつうしんちゅう‥‥{nCTR}{CTR}おまちください！{nCTR}</t>
   </si>
   <si>
-    <t>{NEW}{CTR}Transferring data...{NEW}please wait!{nCTR}</t>
+    <t>{CTR}Transferring data...{NEW}please wait!{nCTR}</t>
   </si>
   <si>
     <t>{CTR}Transfert de données…{NEW}Veuillez patienter!{nCTR}</t>
@@ -2008,7 +2008,7 @@
     <t>ロゴづくりときょうどうアイデアせいさく：{NEW}-Jome{NEW}{NEW}ドットえせいさくしゃ：{NEW}-LJ Birdman</t>
   </si>
   <si>
-    <t>{CTR}Striation City Lab Developers: The Gears of Progress, TimoVM, RisingPhil, EasyAsPi314{nCTR}</t>
+    <t>{CTR}Striation City Lab Developers: {NEW}-The Gears of Progress{NEW}-TimoVM{NEW}-RisingPhil{NEW}-EasyAsPi314{nCTR}</t>
   </si>
   <si>
     <t>Logo et co-créateur:{NEW}-Jome{NEW}{NEW}Spritework:{NEW}-LJ Birdman</t>
@@ -2029,7 +2029,7 @@
     <t>アイコンのドットえせいさくしゃ：{NEW}-LuigiTKO{NEW}-GuiAbel{NEW}-SourAppleとPokémon{NEW}ShowdownやCrystal Clearからの{NEW}アーティストたち</t>
   </si>
   <si>
-    <t>{CTR}Striation City Lab Artists: LJBirdman{NEW}{NEW}Striation City Lab Musicians: AquaticAlloy, Minra Starlight{nCTR}</t>
+    <t>{CTR}Striation City Lab Artists: {NEW}-LJBirdman{NEW}{NEW}Striation City Lab Musicians: {NEW}-AquaticAlloy{NEW}-Minra Starlight{nCTR}</t>
   </si>
   <si>
     <t>Sprites d’icônes: {NEW}-LuigiTKO{NEW}-GuiAbel{NEW}-SourApple{NEW}&amp; les artistes de POKéMON Showdown et Crystal Clear</t>
@@ -2050,7 +2050,7 @@
     <t>リモートとにんいコードじっこうのてつだい：{NEW}{NEW}-TimoVM</t>
   </si>
   <si>
-    <t>{CTR}Striation City Lab Translators: Petros (Japanese), Christobal (Spanish-LA), Lugiadrien (French), Hyd (Portuguese){nCTR}</t>
+    <t>{CTR}Striation City Lab Translators: {NEW}-Petros (Japanese){NEW}-Christobal (Spanish-LA){NEW}-Lugiadrien (French){NEW}-Hyd (Portuguese){nCTR}</t>
   </si>
   <si>
     <t>Support pour l’exécution de code arbitraire à distance:{NEW}-TimoVM</t>
@@ -2106,7 +2106,7 @@
     <t>このライブラリーでビルドできた：{NEW}{NEW}-DevkitPro{NEW}-LibTonc{NEW}-LibGBA</t>
   </si>
   <si>
-    <t>{CTR}Built using:{NEW}-DevkitPro{NEW}-LibTonc{NEW}-LibGBA{nCTR}</t>
+    <t>{CTR}Built using:{NEW}-DevkitPro{NEW}-LibTonc{NEW}{nCTR}</t>
   </si>
   <si>
     <t>Monté avec:{NEW}-DevkitPro{NEW}-LibTonc{NEW}-LibGBA</t>
@@ -6793,6 +6793,9 @@
   </si>
   <si>
     <t>Include Scrolling</t>
+  </si>
+  <si>
+    <t>Vertically Center Text</t>
   </si>
   <si>
     <t>Box Style</t>
@@ -11225,7 +11228,7 @@
       <c r="E85" s="23"/>
       <c r="F85" s="23" t="str">
         <f t="shared" si="2"/>
-        <v>{NEW}Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</v>
+        <v>Poké Transporter GB was sent successfully! You may now power off this GameBoy Advance system.</v>
       </c>
       <c r="G85" s="23" t="s">
         <v>583</v>
@@ -11266,7 +11269,7 @@
       <c r="E86" s="23"/>
       <c r="F86" s="23" t="str">
         <f t="shared" si="2"/>
-        <v>{NEW}An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</v>
+        <v>An error occurred while sending Poké Transporter GB. Press the A button to return to the instructions screen and try again.</v>
       </c>
       <c r="G86" s="23" t="s">
         <v>589</v>
@@ -11411,7 +11414,7 @@
       </c>
       <c r="F89" s="23" t="str">
         <f t="shared" si="2"/>
-        <v>{NEW}{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</v>
+        <v>{CTR}Link was successful!{NEW}Waiting for trade{nCTR}</v>
       </c>
       <c r="G89" s="23" t="s">
         <v>607</v>
@@ -11454,7 +11457,7 @@
       </c>
       <c r="F90" s="23" t="str">
         <f t="shared" si="2"/>
-        <v>{NEW}{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</v>
+        <v>{CTR}Link was successful!{NEW}Waiting for battle{nCTR}</v>
       </c>
       <c r="G90" s="23" t="s">
         <v>613</v>
@@ -11497,7 +11500,7 @@
       </c>
       <c r="F91" s="23" t="str">
         <f t="shared" si="2"/>
-        <v>{NEW}{CTR}Connecting to{NEW}Game Boy{nCTR}</v>
+        <v>{CTR}Connecting to{NEW}Game Boy{nCTR}</v>
       </c>
       <c r="G91" s="23" t="s">
         <v>619</v>
@@ -11540,7 +11543,7 @@
       </c>
       <c r="F92" s="23" t="str">
         <f t="shared" si="2"/>
-        <v>{NEW}{CTR}Transferring data...{NEW}please wait!{nCTR}</v>
+        <v>{CTR}Transferring data...{NEW}please wait!{nCTR}</v>
       </c>
       <c r="G92" s="23" t="s">
         <v>625</v>
@@ -11675,7 +11678,7 @@
       <c r="E95" s="28"/>
       <c r="F95" s="28" t="str">
         <f t="shared" si="2"/>
-        <v>{CTR}Striation City Lab Developers: The Gears of Progress, TimoVM, RisingPhil, EasyAsPi314{nCTR}</v>
+        <v>{CTR}Striation City Lab Developers: {NEW}-The Gears of Progress{NEW}-TimoVM{NEW}-RisingPhil{NEW}-EasyAsPi314{nCTR}</v>
       </c>
       <c r="G95" s="28" t="s">
         <v>644</v>
@@ -11718,7 +11721,7 @@
       <c r="E96" s="28"/>
       <c r="F96" s="28" t="str">
         <f t="shared" si="2"/>
-        <v>{CTR}Striation City Lab Artists: LJBirdman{NEW}{NEW}Striation City Lab Musicians: AquaticAlloy, Minra Starlight{nCTR}</v>
+        <v>{CTR}Striation City Lab Artists: {NEW}-LJBirdman{NEW}{NEW}Striation City Lab Musicians: {NEW}-AquaticAlloy{NEW}-Minra Starlight{nCTR}</v>
       </c>
       <c r="G96" s="28" t="s">
         <v>651</v>
@@ -11761,7 +11764,7 @@
       <c r="E97" s="28"/>
       <c r="F97" s="28" t="str">
         <f t="shared" si="2"/>
-        <v>{CTR}Striation City Lab Translators: Petros (Japanese), Christobal (Spanish-LA), Lugiadrien (French), Hyd (Portuguese){nCTR}</v>
+        <v>{CTR}Striation City Lab Translators: {NEW}-Petros (Japanese){NEW}-Christobal (Spanish-LA){NEW}-Lugiadrien (French){NEW}-Hyd (Portuguese){nCTR}</v>
       </c>
       <c r="G97" s="28" t="s">
         <v>658</v>
@@ -11884,7 +11887,7 @@
       <c r="E100" s="28"/>
       <c r="F100" s="28" t="str">
         <f t="shared" si="2"/>
-        <v>{CTR}Built using:{NEW}-DevkitPro{NEW}-LibTonc{NEW}-LibGBA{nCTR}</v>
+        <v>{CTR}Built using:{NEW}-DevkitPro{NEW}-LibTonc{NEW}{nCTR}</v>
       </c>
       <c r="G100" s="28" t="s">
         <v>676</v>
@@ -26418,6 +26421,9 @@
       <c r="I1" s="56" t="s">
         <v>2242</v>
       </c>
+      <c r="J1" s="56" t="s">
+        <v>2243</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="57" t="s">
@@ -26439,12 +26445,15 @@
         <v>1.0</v>
       </c>
       <c r="G2" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H2" s="59">
         <v>1.0</v>
       </c>
-      <c r="H2" s="59">
+      <c r="I2" s="59">
         <v>0.0</v>
       </c>
-      <c r="I2" s="59">
+      <c r="J2" s="59">
         <v>14.0</v>
       </c>
     </row>
@@ -26468,14 +26477,17 @@
         <v>1.0</v>
       </c>
       <c r="G3" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H3" s="59">
         <v>-1.0</v>
-      </c>
-      <c r="H3" s="59">
-        <v>0.0</v>
       </c>
       <c r="I3" s="59">
         <v>0.0</v>
       </c>
+      <c r="J3" s="59">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="57" t="s">
@@ -26497,12 +26509,15 @@
         <v>0.0</v>
       </c>
       <c r="G4" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H4" s="59">
         <v>-1.0</v>
       </c>
-      <c r="H4" s="59">
+      <c r="I4" s="59">
         <v>0.0</v>
       </c>
-      <c r="I4" s="59">
+      <c r="J4" s="59">
         <v>0.0</v>
       </c>
     </row>
@@ -26526,12 +26541,15 @@
         <v>0.0</v>
       </c>
       <c r="G5" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H5" s="59">
         <v>-1.0</v>
       </c>
-      <c r="H5" s="59">
+      <c r="I5" s="59">
         <v>0.0</v>
       </c>
-      <c r="I5" s="59">
+      <c r="J5" s="59">
         <v>0.0</v>
       </c>
     </row>
@@ -26555,12 +26573,15 @@
         <v>0.0</v>
       </c>
       <c r="G6" s="59">
+        <v>1.0</v>
+      </c>
+      <c r="H6" s="59">
         <v>-1.0</v>
       </c>
-      <c r="H6" s="59">
+      <c r="I6" s="59">
         <v>0.0</v>
       </c>
-      <c r="I6" s="59">
+      <c r="J6" s="59">
         <v>0.0</v>
       </c>
     </row>
@@ -26584,12 +26605,15 @@
         <v>0.0</v>
       </c>
       <c r="G7" s="59">
+        <v>1.0</v>
+      </c>
+      <c r="H7" s="59">
         <v>0.0</v>
       </c>
-      <c r="H7" s="59">
+      <c r="I7" s="59">
         <v>1.0</v>
       </c>
-      <c r="I7" s="59">
+      <c r="J7" s="59">
         <v>1.0</v>
       </c>
     </row>
@@ -26613,12 +26637,15 @@
         <v>0.0</v>
       </c>
       <c r="G8" s="59">
+        <v>1.0</v>
+      </c>
+      <c r="H8" s="59">
         <v>0.0</v>
       </c>
-      <c r="H8" s="59">
+      <c r="I8" s="59">
         <v>4.0</v>
       </c>
-      <c r="I8" s="59">
+      <c r="J8" s="59">
         <v>1.0</v>
       </c>
     </row>
@@ -26642,12 +26669,15 @@
         <v>0.0</v>
       </c>
       <c r="G9" s="59">
+        <v>1.0</v>
+      </c>
+      <c r="H9" s="59">
         <v>0.0</v>
       </c>
-      <c r="H9" s="59">
+      <c r="I9" s="59">
         <v>4.0</v>
       </c>
-      <c r="I9" s="59">
+      <c r="J9" s="59">
         <v>1.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Next verse same as the first
</commit_message>
<xml_diff>
--- a/tools/text_helper/text.xlsx
+++ b/tools/text_helper/text.xlsx
@@ -2029,7 +2029,7 @@
     <t>アイコンのドットえせいさくしゃ：{NEW}-LuigiTKO{NEW}-GuiAbel{NEW}-SourAppleとPokémon{NEW}ShowdownやCrystal Clearからの{NEW}アーティストたち</t>
   </si>
   <si>
-    <t>{CTR}Striation City Lab Artists: {NEW}-LJBirdman{NEW}{NEW}{NEW}Striation City Lab Musicians: {NEW}-AquaticAlloy{NEW}-Minra Starlight{nCTR}</t>
+    <t>{CTR}Striation City Lab Artists: {NEW}-LJBirdman{NEW}{NEW}Striation City Lab Musicians: {NEW}-AquaticAlloy{NEW}-Minra Starlight{nCTR}</t>
   </si>
   <si>
     <t>Sprites d’icônes: {NEW}-LuigiTKO{NEW}-GuiAbel{NEW}-SourApple{NEW}&amp; les artistes de POKéMON Showdown et Crystal Clear</t>
@@ -11721,7 +11721,7 @@
       <c r="E96" s="28"/>
       <c r="F96" s="28" t="str">
         <f t="shared" si="2"/>
-        <v>{CTR}Striation City Lab Artists: {NEW}-LJBirdman{NEW}{NEW}{NEW}Striation City Lab Musicians: {NEW}-AquaticAlloy{NEW}-Minra Starlight{nCTR}</v>
+        <v>{CTR}Striation City Lab Artists: {NEW}-LJBirdman{NEW}{NEW}Striation City Lab Musicians: {NEW}-AquaticAlloy{NEW}-Minra Starlight{nCTR}</v>
       </c>
       <c r="G96" s="28" t="s">
         <v>651</v>

</xml_diff>